<commit_message>
🇸🇾 Update: Syrian cities, Arabic categories, SYP currency
</commit_message>
<xml_diff>
--- a/data/products.xlsx
+++ b/data/products.xlsx
@@ -25,41 +25,33 @@
     <t>price</t>
   </si>
   <si>
-    <t>Toys</t>
+    <t>ألعاب</t>
   </si>
   <si>
-    <t>Clothes</t>
+    <t>ملابس</t>
   </si>
   <si>
-    <t>Perfumes</t>
+    <t>عناية شخصية</t>
   </si>
   <si>
-    <t>Sports</t>
+    <t>رياضة</t>
   </si>
   <si>
-    <t>Home Appliances</t>
+    <t>منزل وديكور</t>
   </si>
   <si>
-    <t>Books</t>
+    <t>كتب</t>
   </si>
   <si>
-    <t>Electronics</t>
+    <t>إلكترونيات</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -75,7 +67,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -83,30 +75,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -405,13 +379,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -423,7 +397,7 @@
         <v>3</v>
       </c>
       <c r="C2">
-        <v>1351</v>
+        <v>193000</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -434,7 +408,7 @@
         <v>3</v>
       </c>
       <c r="C3">
-        <v>874</v>
+        <v>58000</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -445,7 +419,7 @@
         <v>3</v>
       </c>
       <c r="C4">
-        <v>1686</v>
+        <v>36000</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -456,7 +430,7 @@
         <v>4</v>
       </c>
       <c r="C5">
-        <v>1453</v>
+        <v>239000</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -467,7 +441,7 @@
         <v>5</v>
       </c>
       <c r="C6">
-        <v>1215</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -478,7 +452,7 @@
         <v>3</v>
       </c>
       <c r="C7">
-        <v>972</v>
+        <v>92000</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -489,7 +463,7 @@
         <v>5</v>
       </c>
       <c r="C8">
-        <v>1097</v>
+        <v>77000</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -500,7 +474,7 @@
         <v>5</v>
       </c>
       <c r="C9">
-        <v>62</v>
+        <v>55000</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -511,7 +485,7 @@
         <v>5</v>
       </c>
       <c r="C10">
-        <v>1666</v>
+        <v>46000</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -522,7 +496,7 @@
         <v>6</v>
       </c>
       <c r="C11">
-        <v>1298</v>
+        <v>386000</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -533,7 +507,7 @@
         <v>6</v>
       </c>
       <c r="C12">
-        <v>668</v>
+        <v>419000</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -544,7 +518,7 @@
         <v>7</v>
       </c>
       <c r="C13">
-        <v>1540</v>
+        <v>638000</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -555,7 +529,7 @@
         <v>8</v>
       </c>
       <c r="C14">
-        <v>1694</v>
+        <v>21000</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -566,7 +540,7 @@
         <v>3</v>
       </c>
       <c r="C15">
-        <v>177</v>
+        <v>181000</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -577,7 +551,7 @@
         <v>9</v>
       </c>
       <c r="C16">
-        <v>346</v>
+        <v>2228000</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -588,7 +562,7 @@
         <v>5</v>
       </c>
       <c r="C17">
-        <v>1620</v>
+        <v>28000</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -599,7 +573,7 @@
         <v>5</v>
       </c>
       <c r="C18">
-        <v>960</v>
+        <v>27000</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -610,7 +584,7 @@
         <v>4</v>
       </c>
       <c r="C19">
-        <v>1969</v>
+        <v>73000</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -621,7 +595,7 @@
         <v>5</v>
       </c>
       <c r="C20">
-        <v>1186</v>
+        <v>75000</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -632,7 +606,7 @@
         <v>7</v>
       </c>
       <c r="C21">
-        <v>34</v>
+        <v>318000</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -643,7 +617,7 @@
         <v>4</v>
       </c>
       <c r="C22">
-        <v>179</v>
+        <v>179000</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -654,7 +628,7 @@
         <v>9</v>
       </c>
       <c r="C23">
-        <v>1308</v>
+        <v>2965000</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -665,7 +639,7 @@
         <v>5</v>
       </c>
       <c r="C24">
-        <v>1448</v>
+        <v>26000</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -676,7 +650,7 @@
         <v>4</v>
       </c>
       <c r="C25">
-        <v>863</v>
+        <v>193000</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -687,7 +661,7 @@
         <v>3</v>
       </c>
       <c r="C26">
-        <v>1473</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -698,7 +672,7 @@
         <v>3</v>
       </c>
       <c r="C27">
-        <v>139</v>
+        <v>196000</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -709,7 +683,7 @@
         <v>7</v>
       </c>
       <c r="C28">
-        <v>1439</v>
+        <v>798000</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -720,7 +694,7 @@
         <v>6</v>
       </c>
       <c r="C29">
-        <v>1825</v>
+        <v>319000</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -731,7 +705,7 @@
         <v>9</v>
       </c>
       <c r="C30">
-        <v>1279</v>
+        <v>2218000</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -742,7 +716,7 @@
         <v>8</v>
       </c>
       <c r="C31">
-        <v>1648</v>
+        <v>38000</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -753,7 +727,7 @@
         <v>3</v>
       </c>
       <c r="C32">
-        <v>1847</v>
+        <v>144000</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -764,7 +738,7 @@
         <v>8</v>
       </c>
       <c r="C33">
-        <v>74</v>
+        <v>45000</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -775,7 +749,7 @@
         <v>4</v>
       </c>
       <c r="C34">
-        <v>805</v>
+        <v>257000</v>
       </c>
     </row>
     <row r="35" spans="1:3">
@@ -786,7 +760,7 @@
         <v>7</v>
       </c>
       <c r="C35">
-        <v>372</v>
+        <v>86000</v>
       </c>
     </row>
     <row r="36" spans="1:3">
@@ -797,7 +771,7 @@
         <v>4</v>
       </c>
       <c r="C36">
-        <v>286</v>
+        <v>244000</v>
       </c>
     </row>
     <row r="37" spans="1:3">
@@ -808,7 +782,7 @@
         <v>4</v>
       </c>
       <c r="C37">
-        <v>421</v>
+        <v>256000</v>
       </c>
     </row>
     <row r="38" spans="1:3">
@@ -819,7 +793,7 @@
         <v>6</v>
       </c>
       <c r="C38">
-        <v>635</v>
+        <v>121000</v>
       </c>
     </row>
     <row r="39" spans="1:3">
@@ -830,7 +804,7 @@
         <v>7</v>
       </c>
       <c r="C39">
-        <v>1110</v>
+        <v>794000</v>
       </c>
     </row>
     <row r="40" spans="1:3">
@@ -841,7 +815,7 @@
         <v>5</v>
       </c>
       <c r="C40">
-        <v>339</v>
+        <v>128000</v>
       </c>
     </row>
     <row r="41" spans="1:3">
@@ -852,7 +826,7 @@
         <v>7</v>
       </c>
       <c r="C41">
-        <v>1808</v>
+        <v>428000</v>
       </c>
     </row>
     <row r="42" spans="1:3">
@@ -863,7 +837,7 @@
         <v>3</v>
       </c>
       <c r="C42">
-        <v>1574</v>
+        <v>101000</v>
       </c>
     </row>
     <row r="43" spans="1:3">
@@ -874,7 +848,7 @@
         <v>7</v>
       </c>
       <c r="C43">
-        <v>1957</v>
+        <v>239000</v>
       </c>
     </row>
     <row r="44" spans="1:3">
@@ -885,7 +859,7 @@
         <v>9</v>
       </c>
       <c r="C44">
-        <v>1673</v>
+        <v>1381000</v>
       </c>
     </row>
     <row r="45" spans="1:3">
@@ -896,7 +870,7 @@
         <v>8</v>
       </c>
       <c r="C45">
-        <v>1464</v>
+        <v>53000</v>
       </c>
     </row>
     <row r="46" spans="1:3">
@@ -907,7 +881,7 @@
         <v>5</v>
       </c>
       <c r="C46">
-        <v>124</v>
+        <v>46000</v>
       </c>
     </row>
     <row r="47" spans="1:3">
@@ -918,7 +892,7 @@
         <v>8</v>
       </c>
       <c r="C47">
-        <v>427</v>
+        <v>21000</v>
       </c>
     </row>
     <row r="48" spans="1:3">
@@ -929,7 +903,7 @@
         <v>9</v>
       </c>
       <c r="C48">
-        <v>1276</v>
+        <v>2056000</v>
       </c>
     </row>
     <row r="49" spans="1:3">
@@ -940,7 +914,7 @@
         <v>3</v>
       </c>
       <c r="C49">
-        <v>58</v>
+        <v>54000</v>
       </c>
     </row>
     <row r="50" spans="1:3">
@@ -951,7 +925,7 @@
         <v>3</v>
       </c>
       <c r="C50">
-        <v>312</v>
+        <v>121000</v>
       </c>
     </row>
     <row r="51" spans="1:3">
@@ -962,7 +936,7 @@
         <v>3</v>
       </c>
       <c r="C51">
-        <v>1594</v>
+        <v>118000</v>
       </c>
     </row>
     <row r="52" spans="1:3">
@@ -973,7 +947,7 @@
         <v>3</v>
       </c>
       <c r="C52">
-        <v>536</v>
+        <v>184000</v>
       </c>
     </row>
     <row r="53" spans="1:3">
@@ -984,7 +958,7 @@
         <v>3</v>
       </c>
       <c r="C53">
-        <v>747</v>
+        <v>97000</v>
       </c>
     </row>
     <row r="54" spans="1:3">
@@ -995,7 +969,7 @@
         <v>6</v>
       </c>
       <c r="C54">
-        <v>182</v>
+        <v>453000</v>
       </c>
     </row>
     <row r="55" spans="1:3">
@@ -1006,7 +980,7 @@
         <v>6</v>
       </c>
       <c r="C55">
-        <v>637</v>
+        <v>62000</v>
       </c>
     </row>
     <row r="56" spans="1:3">
@@ -1017,7 +991,7 @@
         <v>7</v>
       </c>
       <c r="C56">
-        <v>207</v>
+        <v>550000</v>
       </c>
     </row>
     <row r="57" spans="1:3">
@@ -1028,7 +1002,7 @@
         <v>3</v>
       </c>
       <c r="C57">
-        <v>73</v>
+        <v>167000</v>
       </c>
     </row>
     <row r="58" spans="1:3">
@@ -1039,7 +1013,7 @@
         <v>6</v>
       </c>
       <c r="C58">
-        <v>1017</v>
+        <v>103000</v>
       </c>
     </row>
     <row r="59" spans="1:3">
@@ -1050,7 +1024,7 @@
         <v>7</v>
       </c>
       <c r="C59">
-        <v>794</v>
+        <v>467000</v>
       </c>
     </row>
     <row r="60" spans="1:3">
@@ -1061,7 +1035,7 @@
         <v>9</v>
       </c>
       <c r="C60">
-        <v>421</v>
+        <v>822000</v>
       </c>
     </row>
     <row r="61" spans="1:3">
@@ -1072,7 +1046,7 @@
         <v>6</v>
       </c>
       <c r="C61">
-        <v>1314</v>
+        <v>322000</v>
       </c>
     </row>
     <row r="62" spans="1:3">
@@ -1083,7 +1057,7 @@
         <v>8</v>
       </c>
       <c r="C62">
-        <v>475</v>
+        <v>47000</v>
       </c>
     </row>
     <row r="63" spans="1:3">
@@ -1094,7 +1068,7 @@
         <v>9</v>
       </c>
       <c r="C63">
-        <v>1038</v>
+        <v>1981000</v>
       </c>
     </row>
     <row r="64" spans="1:3">
@@ -1105,7 +1079,7 @@
         <v>3</v>
       </c>
       <c r="C64">
-        <v>1806</v>
+        <v>177000</v>
       </c>
     </row>
     <row r="65" spans="1:3">
@@ -1116,7 +1090,7 @@
         <v>6</v>
       </c>
       <c r="C65">
-        <v>1624</v>
+        <v>138000</v>
       </c>
     </row>
     <row r="66" spans="1:3">
@@ -1127,7 +1101,7 @@
         <v>8</v>
       </c>
       <c r="C66">
-        <v>1432</v>
+        <v>18000</v>
       </c>
     </row>
     <row r="67" spans="1:3">
@@ -1138,7 +1112,7 @@
         <v>3</v>
       </c>
       <c r="C67">
-        <v>1701</v>
+        <v>41000</v>
       </c>
     </row>
     <row r="68" spans="1:3">
@@ -1149,7 +1123,7 @@
         <v>9</v>
       </c>
       <c r="C68">
-        <v>1630</v>
+        <v>1433000</v>
       </c>
     </row>
     <row r="69" spans="1:3">
@@ -1160,7 +1134,7 @@
         <v>5</v>
       </c>
       <c r="C69">
-        <v>1695</v>
+        <v>94000</v>
       </c>
     </row>
     <row r="70" spans="1:3">
@@ -1171,7 +1145,7 @@
         <v>3</v>
       </c>
       <c r="C70">
-        <v>567</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="71" spans="1:3">
@@ -1182,7 +1156,7 @@
         <v>3</v>
       </c>
       <c r="C71">
-        <v>1508</v>
+        <v>89000</v>
       </c>
     </row>
     <row r="72" spans="1:3">
@@ -1193,7 +1167,7 @@
         <v>8</v>
       </c>
       <c r="C72">
-        <v>334</v>
+        <v>22000</v>
       </c>
     </row>
     <row r="73" spans="1:3">
@@ -1204,7 +1178,7 @@
         <v>9</v>
       </c>
       <c r="C73">
-        <v>40</v>
+        <v>2056000</v>
       </c>
     </row>
     <row r="74" spans="1:3">
@@ -1215,7 +1189,7 @@
         <v>8</v>
       </c>
       <c r="C74">
-        <v>1876</v>
+        <v>45000</v>
       </c>
     </row>
     <row r="75" spans="1:3">
@@ -1226,7 +1200,7 @@
         <v>5</v>
       </c>
       <c r="C75">
-        <v>36</v>
+        <v>136000</v>
       </c>
     </row>
     <row r="76" spans="1:3">
@@ -1237,7 +1211,7 @@
         <v>4</v>
       </c>
       <c r="C76">
-        <v>493</v>
+        <v>212000</v>
       </c>
     </row>
     <row r="77" spans="1:3">
@@ -1248,7 +1222,7 @@
         <v>6</v>
       </c>
       <c r="C77">
-        <v>118</v>
+        <v>467000</v>
       </c>
     </row>
     <row r="78" spans="1:3">
@@ -1259,7 +1233,7 @@
         <v>9</v>
       </c>
       <c r="C78">
-        <v>187</v>
+        <v>1994000</v>
       </c>
     </row>
     <row r="79" spans="1:3">
@@ -1270,7 +1244,7 @@
         <v>4</v>
       </c>
       <c r="C79">
-        <v>716</v>
+        <v>91000</v>
       </c>
     </row>
     <row r="80" spans="1:3">
@@ -1281,7 +1255,7 @@
         <v>4</v>
       </c>
       <c r="C80">
-        <v>440</v>
+        <v>144000</v>
       </c>
     </row>
     <row r="81" spans="1:3">
@@ -1292,7 +1266,7 @@
         <v>6</v>
       </c>
       <c r="C81">
-        <v>174</v>
+        <v>221000</v>
       </c>
     </row>
     <row r="82" spans="1:3">
@@ -1303,7 +1277,7 @@
         <v>3</v>
       </c>
       <c r="C82">
-        <v>734</v>
+        <v>83000</v>
       </c>
     </row>
     <row r="83" spans="1:3">
@@ -1314,7 +1288,7 @@
         <v>8</v>
       </c>
       <c r="C83">
-        <v>1689</v>
+        <v>44000</v>
       </c>
     </row>
     <row r="84" spans="1:3">
@@ -1325,7 +1299,7 @@
         <v>8</v>
       </c>
       <c r="C84">
-        <v>352</v>
+        <v>19000</v>
       </c>
     </row>
     <row r="85" spans="1:3">
@@ -1336,7 +1310,7 @@
         <v>8</v>
       </c>
       <c r="C85">
-        <v>77</v>
+        <v>31000</v>
       </c>
     </row>
     <row r="86" spans="1:3">
@@ -1347,7 +1321,7 @@
         <v>8</v>
       </c>
       <c r="C86">
-        <v>1017</v>
+        <v>78000</v>
       </c>
     </row>
     <row r="87" spans="1:3">
@@ -1358,7 +1332,7 @@
         <v>6</v>
       </c>
       <c r="C87">
-        <v>205</v>
+        <v>413000</v>
       </c>
     </row>
     <row r="88" spans="1:3">
@@ -1369,7 +1343,7 @@
         <v>6</v>
       </c>
       <c r="C88">
-        <v>1636</v>
+        <v>165000</v>
       </c>
     </row>
     <row r="89" spans="1:3">
@@ -1380,7 +1354,7 @@
         <v>8</v>
       </c>
       <c r="C89">
-        <v>1404</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="90" spans="1:3">
@@ -1391,7 +1365,7 @@
         <v>6</v>
       </c>
       <c r="C90">
-        <v>522</v>
+        <v>276000</v>
       </c>
     </row>
     <row r="91" spans="1:3">
@@ -1402,7 +1376,7 @@
         <v>6</v>
       </c>
       <c r="C91">
-        <v>418</v>
+        <v>234000</v>
       </c>
     </row>
     <row r="92" spans="1:3">
@@ -1413,7 +1387,7 @@
         <v>7</v>
       </c>
       <c r="C92">
-        <v>72</v>
+        <v>356000</v>
       </c>
     </row>
     <row r="93" spans="1:3">
@@ -1424,7 +1398,7 @@
         <v>6</v>
       </c>
       <c r="C93">
-        <v>1180</v>
+        <v>367000</v>
       </c>
     </row>
     <row r="94" spans="1:3">
@@ -1435,7 +1409,7 @@
         <v>8</v>
       </c>
       <c r="C94">
-        <v>1949</v>
+        <v>38000</v>
       </c>
     </row>
     <row r="95" spans="1:3">
@@ -1446,7 +1420,7 @@
         <v>4</v>
       </c>
       <c r="C95">
-        <v>594</v>
+        <v>225000</v>
       </c>
     </row>
     <row r="96" spans="1:3">
@@ -1457,7 +1431,7 @@
         <v>5</v>
       </c>
       <c r="C96">
-        <v>1238</v>
+        <v>103000</v>
       </c>
     </row>
     <row r="97" spans="1:3">
@@ -1468,7 +1442,7 @@
         <v>3</v>
       </c>
       <c r="C97">
-        <v>998</v>
+        <v>44000</v>
       </c>
     </row>
     <row r="98" spans="1:3">
@@ -1479,7 +1453,7 @@
         <v>7</v>
       </c>
       <c r="C98">
-        <v>1701</v>
+        <v>314000</v>
       </c>
     </row>
     <row r="99" spans="1:3">
@@ -1490,7 +1464,7 @@
         <v>6</v>
       </c>
       <c r="C99">
-        <v>956</v>
+        <v>460000</v>
       </c>
     </row>
     <row r="100" spans="1:3">
@@ -1501,7 +1475,7 @@
         <v>4</v>
       </c>
       <c r="C100">
-        <v>1462</v>
+        <v>58000</v>
       </c>
     </row>
     <row r="101" spans="1:3">
@@ -1512,7 +1486,7 @@
         <v>8</v>
       </c>
       <c r="C101">
-        <v>1333</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="102" spans="1:3">
@@ -1523,7 +1497,7 @@
         <v>6</v>
       </c>
       <c r="C102">
-        <v>662</v>
+        <v>245000</v>
       </c>
     </row>
     <row r="103" spans="1:3">
@@ -1534,7 +1508,7 @@
         <v>7</v>
       </c>
       <c r="C103">
-        <v>953</v>
+        <v>354000</v>
       </c>
     </row>
     <row r="104" spans="1:3">
@@ -1545,7 +1519,7 @@
         <v>3</v>
       </c>
       <c r="C104">
-        <v>1531</v>
+        <v>46000</v>
       </c>
     </row>
     <row r="105" spans="1:3">
@@ -1556,7 +1530,7 @@
         <v>3</v>
       </c>
       <c r="C105">
-        <v>1025</v>
+        <v>84000</v>
       </c>
     </row>
     <row r="106" spans="1:3">
@@ -1567,7 +1541,7 @@
         <v>8</v>
       </c>
       <c r="C106">
-        <v>1046</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="107" spans="1:3">
@@ -1578,7 +1552,7 @@
         <v>6</v>
       </c>
       <c r="C107">
-        <v>831</v>
+        <v>148000</v>
       </c>
     </row>
     <row r="108" spans="1:3">
@@ -1589,7 +1563,7 @@
         <v>4</v>
       </c>
       <c r="C108">
-        <v>235</v>
+        <v>217000</v>
       </c>
     </row>
     <row r="109" spans="1:3">
@@ -1600,7 +1574,7 @@
         <v>5</v>
       </c>
       <c r="C109">
-        <v>804</v>
+        <v>147000</v>
       </c>
     </row>
     <row r="110" spans="1:3">
@@ -1611,7 +1585,7 @@
         <v>8</v>
       </c>
       <c r="C110">
-        <v>217</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="111" spans="1:3">
@@ -1622,7 +1596,7 @@
         <v>5</v>
       </c>
       <c r="C111">
-        <v>90</v>
+        <v>137000</v>
       </c>
     </row>
     <row r="112" spans="1:3">
@@ -1633,7 +1607,7 @@
         <v>3</v>
       </c>
       <c r="C112">
-        <v>173</v>
+        <v>66000</v>
       </c>
     </row>
     <row r="113" spans="1:3">
@@ -1644,7 +1618,7 @@
         <v>7</v>
       </c>
       <c r="C113">
-        <v>1592</v>
+        <v>351000</v>
       </c>
     </row>
     <row r="114" spans="1:3">
@@ -1655,7 +1629,7 @@
         <v>8</v>
       </c>
       <c r="C114">
-        <v>1373</v>
+        <v>27000</v>
       </c>
     </row>
     <row r="115" spans="1:3">
@@ -1666,7 +1640,7 @@
         <v>9</v>
       </c>
       <c r="C115">
-        <v>229</v>
+        <v>1510000</v>
       </c>
     </row>
     <row r="116" spans="1:3">
@@ -1677,7 +1651,7 @@
         <v>6</v>
       </c>
       <c r="C116">
-        <v>1237</v>
+        <v>421000</v>
       </c>
     </row>
     <row r="117" spans="1:3">
@@ -1688,7 +1662,7 @@
         <v>3</v>
       </c>
       <c r="C117">
-        <v>491</v>
+        <v>173000</v>
       </c>
     </row>
     <row r="118" spans="1:3">
@@ -1699,7 +1673,7 @@
         <v>4</v>
       </c>
       <c r="C118">
-        <v>1956</v>
+        <v>187000</v>
       </c>
     </row>
     <row r="119" spans="1:3">
@@ -1710,7 +1684,7 @@
         <v>5</v>
       </c>
       <c r="C119">
-        <v>1778</v>
+        <v>87000</v>
       </c>
     </row>
     <row r="120" spans="1:3">
@@ -1721,7 +1695,7 @@
         <v>6</v>
       </c>
       <c r="C120">
-        <v>1079</v>
+        <v>422000</v>
       </c>
     </row>
     <row r="121" spans="1:3">
@@ -1732,7 +1706,7 @@
         <v>9</v>
       </c>
       <c r="C121">
-        <v>924</v>
+        <v>2894000</v>
       </c>
     </row>
     <row r="122" spans="1:3">
@@ -1743,7 +1717,7 @@
         <v>8</v>
       </c>
       <c r="C122">
-        <v>1810</v>
+        <v>64000</v>
       </c>
     </row>
     <row r="123" spans="1:3">
@@ -1754,7 +1728,7 @@
         <v>3</v>
       </c>
       <c r="C123">
-        <v>532</v>
+        <v>179000</v>
       </c>
     </row>
     <row r="124" spans="1:3">
@@ -1765,7 +1739,7 @@
         <v>4</v>
       </c>
       <c r="C124">
-        <v>614</v>
+        <v>152000</v>
       </c>
     </row>
     <row r="125" spans="1:3">
@@ -1776,7 +1750,7 @@
         <v>3</v>
       </c>
       <c r="C125">
-        <v>1344</v>
+        <v>122000</v>
       </c>
     </row>
     <row r="126" spans="1:3">
@@ -1787,7 +1761,7 @@
         <v>8</v>
       </c>
       <c r="C126">
-        <v>1601</v>
+        <v>38000</v>
       </c>
     </row>
     <row r="127" spans="1:3">
@@ -1798,7 +1772,7 @@
         <v>9</v>
       </c>
       <c r="C127">
-        <v>1929</v>
+        <v>1066000</v>
       </c>
     </row>
     <row r="128" spans="1:3">
@@ -1809,7 +1783,7 @@
         <v>6</v>
       </c>
       <c r="C128">
-        <v>1787</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="129" spans="1:3">
@@ -1820,7 +1794,7 @@
         <v>9</v>
       </c>
       <c r="C129">
-        <v>1276</v>
+        <v>2521000</v>
       </c>
     </row>
     <row r="130" spans="1:3">
@@ -1831,7 +1805,7 @@
         <v>7</v>
       </c>
       <c r="C130">
-        <v>1485</v>
+        <v>173000</v>
       </c>
     </row>
     <row r="131" spans="1:3">
@@ -1842,7 +1816,7 @@
         <v>5</v>
       </c>
       <c r="C131">
-        <v>1570</v>
+        <v>32000</v>
       </c>
     </row>
     <row r="132" spans="1:3">
@@ -1853,7 +1827,7 @@
         <v>8</v>
       </c>
       <c r="C132">
-        <v>1769</v>
+        <v>24000</v>
       </c>
     </row>
     <row r="133" spans="1:3">
@@ -1864,7 +1838,7 @@
         <v>4</v>
       </c>
       <c r="C133">
-        <v>1631</v>
+        <v>89000</v>
       </c>
     </row>
     <row r="134" spans="1:3">
@@ -1875,7 +1849,7 @@
         <v>3</v>
       </c>
       <c r="C134">
-        <v>695</v>
+        <v>190000</v>
       </c>
     </row>
     <row r="135" spans="1:3">
@@ -1886,7 +1860,7 @@
         <v>5</v>
       </c>
       <c r="C135">
-        <v>635</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="136" spans="1:3">
@@ -1897,7 +1871,7 @@
         <v>4</v>
       </c>
       <c r="C136">
-        <v>1158</v>
+        <v>252000</v>
       </c>
     </row>
     <row r="137" spans="1:3">
@@ -1908,7 +1882,7 @@
         <v>9</v>
       </c>
       <c r="C137">
-        <v>1786</v>
+        <v>2229000</v>
       </c>
     </row>
     <row r="138" spans="1:3">
@@ -1919,7 +1893,7 @@
         <v>9</v>
       </c>
       <c r="C138">
-        <v>1637</v>
+        <v>2942000</v>
       </c>
     </row>
     <row r="139" spans="1:3">
@@ -1930,7 +1904,7 @@
         <v>6</v>
       </c>
       <c r="C139">
-        <v>1066</v>
+        <v>72000</v>
       </c>
     </row>
     <row r="140" spans="1:3">
@@ -1941,7 +1915,7 @@
         <v>5</v>
       </c>
       <c r="C140">
-        <v>1516</v>
+        <v>118000</v>
       </c>
     </row>
     <row r="141" spans="1:3">
@@ -1952,7 +1926,7 @@
         <v>8</v>
       </c>
       <c r="C141">
-        <v>44</v>
+        <v>58000</v>
       </c>
     </row>
     <row r="142" spans="1:3">
@@ -1963,7 +1937,7 @@
         <v>4</v>
       </c>
       <c r="C142">
-        <v>1722</v>
+        <v>202000</v>
       </c>
     </row>
     <row r="143" spans="1:3">
@@ -1974,7 +1948,7 @@
         <v>3</v>
       </c>
       <c r="C143">
-        <v>1518</v>
+        <v>149000</v>
       </c>
     </row>
     <row r="144" spans="1:3">
@@ -1985,7 +1959,7 @@
         <v>3</v>
       </c>
       <c r="C144">
-        <v>1009</v>
+        <v>165000</v>
       </c>
     </row>
     <row r="145" spans="1:3">
@@ -1996,7 +1970,7 @@
         <v>6</v>
       </c>
       <c r="C145">
-        <v>1048</v>
+        <v>168000</v>
       </c>
     </row>
     <row r="146" spans="1:3">
@@ -2007,7 +1981,7 @@
         <v>3</v>
       </c>
       <c r="C146">
-        <v>1020</v>
+        <v>171000</v>
       </c>
     </row>
     <row r="147" spans="1:3">
@@ -2018,7 +1992,7 @@
         <v>8</v>
       </c>
       <c r="C147">
-        <v>566</v>
+        <v>11000</v>
       </c>
     </row>
     <row r="148" spans="1:3">
@@ -2029,7 +2003,7 @@
         <v>5</v>
       </c>
       <c r="C148">
-        <v>380</v>
+        <v>49000</v>
       </c>
     </row>
     <row r="149" spans="1:3">
@@ -2040,7 +2014,7 @@
         <v>5</v>
       </c>
       <c r="C149">
-        <v>1506</v>
+        <v>88000</v>
       </c>
     </row>
     <row r="150" spans="1:3">
@@ -2051,7 +2025,7 @@
         <v>9</v>
       </c>
       <c r="C150">
-        <v>20</v>
+        <v>1893000</v>
       </c>
     </row>
     <row r="151" spans="1:3">
@@ -2062,7 +2036,7 @@
         <v>5</v>
       </c>
       <c r="C151">
-        <v>337</v>
+        <v>48000</v>
       </c>
     </row>
     <row r="152" spans="1:3">
@@ -2073,7 +2047,7 @@
         <v>5</v>
       </c>
       <c r="C152">
-        <v>1000</v>
+        <v>95000</v>
       </c>
     </row>
     <row r="153" spans="1:3">
@@ -2084,7 +2058,7 @@
         <v>9</v>
       </c>
       <c r="C153">
-        <v>673</v>
+        <v>2280000</v>
       </c>
     </row>
     <row r="154" spans="1:3">
@@ -2095,7 +2069,7 @@
         <v>4</v>
       </c>
       <c r="C154">
-        <v>1120</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="155" spans="1:3">
@@ -2106,7 +2080,7 @@
         <v>9</v>
       </c>
       <c r="C155">
-        <v>1195</v>
+        <v>2358000</v>
       </c>
     </row>
     <row r="156" spans="1:3">
@@ -2117,7 +2091,7 @@
         <v>5</v>
       </c>
       <c r="C156">
-        <v>178</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="157" spans="1:3">
@@ -2128,7 +2102,7 @@
         <v>5</v>
       </c>
       <c r="C157">
-        <v>1183</v>
+        <v>87000</v>
       </c>
     </row>
     <row r="158" spans="1:3">
@@ -2139,7 +2113,7 @@
         <v>6</v>
       </c>
       <c r="C158">
-        <v>1289</v>
+        <v>296000</v>
       </c>
     </row>
     <row r="159" spans="1:3">
@@ -2150,7 +2124,7 @@
         <v>5</v>
       </c>
       <c r="C159">
-        <v>235</v>
+        <v>65000</v>
       </c>
     </row>
     <row r="160" spans="1:3">
@@ -2161,7 +2135,7 @@
         <v>7</v>
       </c>
       <c r="C160">
-        <v>21</v>
+        <v>599000</v>
       </c>
     </row>
     <row r="161" spans="1:3">
@@ -2172,7 +2146,7 @@
         <v>7</v>
       </c>
       <c r="C161">
-        <v>124</v>
+        <v>188000</v>
       </c>
     </row>
     <row r="162" spans="1:3">
@@ -2183,7 +2157,7 @@
         <v>9</v>
       </c>
       <c r="C162">
-        <v>1153</v>
+        <v>1722000</v>
       </c>
     </row>
     <row r="163" spans="1:3">
@@ -2194,7 +2168,7 @@
         <v>8</v>
       </c>
       <c r="C163">
-        <v>1765</v>
+        <v>74000</v>
       </c>
     </row>
     <row r="164" spans="1:3">
@@ -2205,7 +2179,7 @@
         <v>6</v>
       </c>
       <c r="C164">
-        <v>1189</v>
+        <v>351000</v>
       </c>
     </row>
     <row r="165" spans="1:3">
@@ -2216,7 +2190,7 @@
         <v>7</v>
       </c>
       <c r="C165">
-        <v>1497</v>
+        <v>283000</v>
       </c>
     </row>
     <row r="166" spans="1:3">
@@ -2227,7 +2201,7 @@
         <v>6</v>
       </c>
       <c r="C166">
-        <v>848</v>
+        <v>118000</v>
       </c>
     </row>
     <row r="167" spans="1:3">
@@ -2238,7 +2212,7 @@
         <v>8</v>
       </c>
       <c r="C167">
-        <v>924</v>
+        <v>57000</v>
       </c>
     </row>
     <row r="168" spans="1:3">
@@ -2249,7 +2223,7 @@
         <v>7</v>
       </c>
       <c r="C168">
-        <v>903</v>
+        <v>245000</v>
       </c>
     </row>
     <row r="169" spans="1:3">
@@ -2260,7 +2234,7 @@
         <v>8</v>
       </c>
       <c r="C169">
-        <v>376</v>
+        <v>79000</v>
       </c>
     </row>
     <row r="170" spans="1:3">
@@ -2271,7 +2245,7 @@
         <v>6</v>
       </c>
       <c r="C170">
-        <v>669</v>
+        <v>438000</v>
       </c>
     </row>
     <row r="171" spans="1:3">
@@ -2282,7 +2256,7 @@
         <v>8</v>
       </c>
       <c r="C171">
-        <v>1104</v>
+        <v>77000</v>
       </c>
     </row>
     <row r="172" spans="1:3">
@@ -2293,7 +2267,7 @@
         <v>5</v>
       </c>
       <c r="C172">
-        <v>808</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="173" spans="1:3">
@@ -2304,7 +2278,7 @@
         <v>3</v>
       </c>
       <c r="C173">
-        <v>1289</v>
+        <v>183000</v>
       </c>
     </row>
     <row r="174" spans="1:3">
@@ -2315,7 +2289,7 @@
         <v>7</v>
       </c>
       <c r="C174">
-        <v>1167</v>
+        <v>411000</v>
       </c>
     </row>
     <row r="175" spans="1:3">
@@ -2326,7 +2300,7 @@
         <v>5</v>
       </c>
       <c r="C175">
-        <v>1623</v>
+        <v>145000</v>
       </c>
     </row>
     <row r="176" spans="1:3">
@@ -2337,7 +2311,7 @@
         <v>6</v>
       </c>
       <c r="C176">
-        <v>1924</v>
+        <v>49000</v>
       </c>
     </row>
     <row r="177" spans="1:3">
@@ -2348,7 +2322,7 @@
         <v>7</v>
       </c>
       <c r="C177">
-        <v>1485</v>
+        <v>194000</v>
       </c>
     </row>
     <row r="178" spans="1:3">
@@ -2359,7 +2333,7 @@
         <v>3</v>
       </c>
       <c r="C178">
-        <v>1624</v>
+        <v>122000</v>
       </c>
     </row>
     <row r="179" spans="1:3">
@@ -2370,7 +2344,7 @@
         <v>7</v>
       </c>
       <c r="C179">
-        <v>988</v>
+        <v>394000</v>
       </c>
     </row>
     <row r="180" spans="1:3">
@@ -2381,7 +2355,7 @@
         <v>4</v>
       </c>
       <c r="C180">
-        <v>771</v>
+        <v>111000</v>
       </c>
     </row>
     <row r="181" spans="1:3">
@@ -2392,7 +2366,7 @@
         <v>3</v>
       </c>
       <c r="C181">
-        <v>1492</v>
+        <v>44000</v>
       </c>
     </row>
     <row r="182" spans="1:3">
@@ -2403,7 +2377,7 @@
         <v>3</v>
       </c>
       <c r="C182">
-        <v>913</v>
+        <v>91000</v>
       </c>
     </row>
     <row r="183" spans="1:3">
@@ -2414,7 +2388,7 @@
         <v>7</v>
       </c>
       <c r="C183">
-        <v>386</v>
+        <v>660000</v>
       </c>
     </row>
     <row r="184" spans="1:3">
@@ -2425,7 +2399,7 @@
         <v>3</v>
       </c>
       <c r="C184">
-        <v>1130</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="185" spans="1:3">
@@ -2436,7 +2410,7 @@
         <v>3</v>
       </c>
       <c r="C185">
-        <v>850</v>
+        <v>51000</v>
       </c>
     </row>
     <row r="186" spans="1:3">
@@ -2447,7 +2421,7 @@
         <v>7</v>
       </c>
       <c r="C186">
-        <v>42</v>
+        <v>577000</v>
       </c>
     </row>
     <row r="187" spans="1:3">
@@ -2458,7 +2432,7 @@
         <v>6</v>
       </c>
       <c r="C187">
-        <v>1100</v>
+        <v>457000</v>
       </c>
     </row>
     <row r="188" spans="1:3">
@@ -2469,7 +2443,7 @@
         <v>6</v>
       </c>
       <c r="C188">
-        <v>1054</v>
+        <v>75000</v>
       </c>
     </row>
     <row r="189" spans="1:3">
@@ -2480,7 +2454,7 @@
         <v>6</v>
       </c>
       <c r="C189">
-        <v>44</v>
+        <v>429000</v>
       </c>
     </row>
     <row r="190" spans="1:3">
@@ -2491,7 +2465,7 @@
         <v>8</v>
       </c>
       <c r="C190">
-        <v>1770</v>
+        <v>78000</v>
       </c>
     </row>
     <row r="191" spans="1:3">
@@ -2502,7 +2476,7 @@
         <v>7</v>
       </c>
       <c r="C191">
-        <v>887</v>
+        <v>208000</v>
       </c>
     </row>
     <row r="192" spans="1:3">
@@ -2513,7 +2487,7 @@
         <v>8</v>
       </c>
       <c r="C192">
-        <v>1352</v>
+        <v>26000</v>
       </c>
     </row>
     <row r="193" spans="1:3">
@@ -2524,7 +2498,7 @@
         <v>9</v>
       </c>
       <c r="C193">
-        <v>1860</v>
+        <v>2446000</v>
       </c>
     </row>
     <row r="194" spans="1:3">
@@ -2535,7 +2509,7 @@
         <v>3</v>
       </c>
       <c r="C194">
-        <v>1246</v>
+        <v>170000</v>
       </c>
     </row>
     <row r="195" spans="1:3">
@@ -2546,7 +2520,7 @@
         <v>6</v>
       </c>
       <c r="C195">
-        <v>1256</v>
+        <v>124000</v>
       </c>
     </row>
     <row r="196" spans="1:3">
@@ -2557,7 +2531,7 @@
         <v>9</v>
       </c>
       <c r="C196">
-        <v>956</v>
+        <v>1585000</v>
       </c>
     </row>
     <row r="197" spans="1:3">
@@ -2568,7 +2542,7 @@
         <v>8</v>
       </c>
       <c r="C197">
-        <v>1213</v>
+        <v>77000</v>
       </c>
     </row>
     <row r="198" spans="1:3">
@@ -2579,7 +2553,7 @@
         <v>7</v>
       </c>
       <c r="C198">
-        <v>1953</v>
+        <v>701000</v>
       </c>
     </row>
     <row r="199" spans="1:3">
@@ -2590,7 +2564,7 @@
         <v>9</v>
       </c>
       <c r="C199">
-        <v>922</v>
+        <v>2233000</v>
       </c>
     </row>
     <row r="200" spans="1:3">
@@ -2601,7 +2575,7 @@
         <v>6</v>
       </c>
       <c r="C200">
-        <v>1123</v>
+        <v>148000</v>
       </c>
     </row>
     <row r="201" spans="1:3">
@@ -2612,7 +2586,7 @@
         <v>8</v>
       </c>
       <c r="C201">
-        <v>413</v>
+        <v>79000</v>
       </c>
     </row>
     <row r="202" spans="1:3">
@@ -2623,7 +2597,7 @@
         <v>4</v>
       </c>
       <c r="C202">
-        <v>1441</v>
+        <v>243000</v>
       </c>
     </row>
     <row r="203" spans="1:3">
@@ -2634,7 +2608,7 @@
         <v>5</v>
       </c>
       <c r="C203">
-        <v>1410</v>
+        <v>71000</v>
       </c>
     </row>
     <row r="204" spans="1:3">
@@ -2645,7 +2619,7 @@
         <v>4</v>
       </c>
       <c r="C204">
-        <v>252</v>
+        <v>232000</v>
       </c>
     </row>
     <row r="205" spans="1:3">
@@ -2656,7 +2630,7 @@
         <v>9</v>
       </c>
       <c r="C205">
-        <v>443</v>
+        <v>1776000</v>
       </c>
     </row>
     <row r="206" spans="1:3">
@@ -2667,7 +2641,7 @@
         <v>8</v>
       </c>
       <c r="C206">
-        <v>675</v>
+        <v>61000</v>
       </c>
     </row>
     <row r="207" spans="1:3">
@@ -2678,7 +2652,7 @@
         <v>9</v>
       </c>
       <c r="C207">
-        <v>631</v>
+        <v>2029000</v>
       </c>
     </row>
     <row r="208" spans="1:3">
@@ -2689,7 +2663,7 @@
         <v>3</v>
       </c>
       <c r="C208">
-        <v>279</v>
+        <v>142000</v>
       </c>
     </row>
     <row r="209" spans="1:3">
@@ -2700,7 +2674,7 @@
         <v>8</v>
       </c>
       <c r="C209">
-        <v>1400</v>
+        <v>76000</v>
       </c>
     </row>
     <row r="210" spans="1:3">
@@ -2711,7 +2685,7 @@
         <v>7</v>
       </c>
       <c r="C210">
-        <v>1463</v>
+        <v>542000</v>
       </c>
     </row>
     <row r="211" spans="1:3">
@@ -2722,7 +2696,7 @@
         <v>9</v>
       </c>
       <c r="C211">
-        <v>918</v>
+        <v>995000</v>
       </c>
     </row>
     <row r="212" spans="1:3">
@@ -2733,7 +2707,7 @@
         <v>7</v>
       </c>
       <c r="C212">
-        <v>1622</v>
+        <v>333000</v>
       </c>
     </row>
     <row r="213" spans="1:3">
@@ -2744,7 +2718,7 @@
         <v>6</v>
       </c>
       <c r="C213">
-        <v>1024</v>
+        <v>155000</v>
       </c>
     </row>
     <row r="214" spans="1:3">
@@ -2755,7 +2729,7 @@
         <v>5</v>
       </c>
       <c r="C214">
-        <v>867</v>
+        <v>36000</v>
       </c>
     </row>
     <row r="215" spans="1:3">
@@ -2766,7 +2740,7 @@
         <v>6</v>
       </c>
       <c r="C215">
-        <v>1822</v>
+        <v>213000</v>
       </c>
     </row>
     <row r="216" spans="1:3">
@@ -2777,7 +2751,7 @@
         <v>9</v>
       </c>
       <c r="C216">
-        <v>1805</v>
+        <v>586000</v>
       </c>
     </row>
     <row r="217" spans="1:3">
@@ -2788,7 +2762,7 @@
         <v>4</v>
       </c>
       <c r="C217">
-        <v>257</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="218" spans="1:3">
@@ -2799,7 +2773,7 @@
         <v>4</v>
       </c>
       <c r="C218">
-        <v>1870</v>
+        <v>191000</v>
       </c>
     </row>
     <row r="219" spans="1:3">
@@ -2810,7 +2784,7 @@
         <v>8</v>
       </c>
       <c r="C219">
-        <v>565</v>
+        <v>39000</v>
       </c>
     </row>
     <row r="220" spans="1:3">
@@ -2821,7 +2795,7 @@
         <v>3</v>
       </c>
       <c r="C220">
-        <v>68</v>
+        <v>180000</v>
       </c>
     </row>
     <row r="221" spans="1:3">
@@ -2832,7 +2806,7 @@
         <v>9</v>
       </c>
       <c r="C221">
-        <v>896</v>
+        <v>1402000</v>
       </c>
     </row>
     <row r="222" spans="1:3">
@@ -2843,7 +2817,7 @@
         <v>5</v>
       </c>
       <c r="C222">
-        <v>117</v>
+        <v>21000</v>
       </c>
     </row>
     <row r="223" spans="1:3">
@@ -2854,7 +2828,7 @@
         <v>5</v>
       </c>
       <c r="C223">
-        <v>1193</v>
+        <v>38000</v>
       </c>
     </row>
     <row r="224" spans="1:3">
@@ -2865,7 +2839,7 @@
         <v>6</v>
       </c>
       <c r="C224">
-        <v>1969</v>
+        <v>402000</v>
       </c>
     </row>
     <row r="225" spans="1:3">
@@ -2876,7 +2850,7 @@
         <v>7</v>
       </c>
       <c r="C225">
-        <v>1905</v>
+        <v>726000</v>
       </c>
     </row>
     <row r="226" spans="1:3">
@@ -2887,7 +2861,7 @@
         <v>4</v>
       </c>
       <c r="C226">
-        <v>154</v>
+        <v>65000</v>
       </c>
     </row>
     <row r="227" spans="1:3">
@@ -2898,7 +2872,7 @@
         <v>7</v>
       </c>
       <c r="C227">
-        <v>995</v>
+        <v>314000</v>
       </c>
     </row>
     <row r="228" spans="1:3">
@@ -2909,7 +2883,7 @@
         <v>8</v>
       </c>
       <c r="C228">
-        <v>1097</v>
+        <v>18000</v>
       </c>
     </row>
     <row r="229" spans="1:3">
@@ -2920,7 +2894,7 @@
         <v>7</v>
       </c>
       <c r="C229">
-        <v>1394</v>
+        <v>112000</v>
       </c>
     </row>
     <row r="230" spans="1:3">
@@ -2931,7 +2905,7 @@
         <v>4</v>
       </c>
       <c r="C230">
-        <v>1573</v>
+        <v>270000</v>
       </c>
     </row>
     <row r="231" spans="1:3">
@@ -2942,7 +2916,7 @@
         <v>3</v>
       </c>
       <c r="C231">
-        <v>1936</v>
+        <v>114000</v>
       </c>
     </row>
     <row r="232" spans="1:3">
@@ -2953,7 +2927,7 @@
         <v>3</v>
       </c>
       <c r="C232">
-        <v>475</v>
+        <v>48000</v>
       </c>
     </row>
     <row r="233" spans="1:3">
@@ -2964,7 +2938,7 @@
         <v>5</v>
       </c>
       <c r="C233">
-        <v>243</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="234" spans="1:3">
@@ -2975,7 +2949,7 @@
         <v>3</v>
       </c>
       <c r="C234">
-        <v>1441</v>
+        <v>101000</v>
       </c>
     </row>
     <row r="235" spans="1:3">
@@ -2986,7 +2960,7 @@
         <v>4</v>
       </c>
       <c r="C235">
-        <v>1298</v>
+        <v>221000</v>
       </c>
     </row>
     <row r="236" spans="1:3">
@@ -2997,7 +2971,7 @@
         <v>5</v>
       </c>
       <c r="C236">
-        <v>1749</v>
+        <v>144000</v>
       </c>
     </row>
     <row r="237" spans="1:3">
@@ -3008,7 +2982,7 @@
         <v>5</v>
       </c>
       <c r="C237">
-        <v>537</v>
+        <v>74000</v>
       </c>
     </row>
     <row r="238" spans="1:3">
@@ -3019,7 +2993,7 @@
         <v>8</v>
       </c>
       <c r="C238">
-        <v>1262</v>
+        <v>79000</v>
       </c>
     </row>
     <row r="239" spans="1:3">
@@ -3030,7 +3004,7 @@
         <v>6</v>
       </c>
       <c r="C239">
-        <v>1829</v>
+        <v>107000</v>
       </c>
     </row>
     <row r="240" spans="1:3">
@@ -3041,7 +3015,7 @@
         <v>8</v>
       </c>
       <c r="C240">
-        <v>1458</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="241" spans="1:3">
@@ -3052,7 +3026,7 @@
         <v>8</v>
       </c>
       <c r="C241">
-        <v>311</v>
+        <v>41000</v>
       </c>
     </row>
     <row r="242" spans="1:3">
@@ -3063,7 +3037,7 @@
         <v>6</v>
       </c>
       <c r="C242">
-        <v>1829</v>
+        <v>441000</v>
       </c>
     </row>
     <row r="243" spans="1:3">
@@ -3074,7 +3048,7 @@
         <v>8</v>
       </c>
       <c r="C243">
-        <v>387</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="244" spans="1:3">
@@ -3085,7 +3059,7 @@
         <v>3</v>
       </c>
       <c r="C244">
-        <v>1640</v>
+        <v>134000</v>
       </c>
     </row>
     <row r="245" spans="1:3">
@@ -3096,7 +3070,7 @@
         <v>6</v>
       </c>
       <c r="C245">
-        <v>876</v>
+        <v>137000</v>
       </c>
     </row>
     <row r="246" spans="1:3">
@@ -3107,7 +3081,7 @@
         <v>4</v>
       </c>
       <c r="C246">
-        <v>841</v>
+        <v>74000</v>
       </c>
     </row>
     <row r="247" spans="1:3">
@@ -3118,7 +3092,7 @@
         <v>5</v>
       </c>
       <c r="C247">
-        <v>935</v>
+        <v>44000</v>
       </c>
     </row>
     <row r="248" spans="1:3">
@@ -3129,7 +3103,7 @@
         <v>5</v>
       </c>
       <c r="C248">
-        <v>814</v>
+        <v>130000</v>
       </c>
     </row>
     <row r="249" spans="1:3">
@@ -3140,7 +3114,7 @@
         <v>9</v>
       </c>
       <c r="C249">
-        <v>1300</v>
+        <v>1951000</v>
       </c>
     </row>
     <row r="250" spans="1:3">
@@ -3151,7 +3125,7 @@
         <v>4</v>
       </c>
       <c r="C250">
-        <v>283</v>
+        <v>158000</v>
       </c>
     </row>
     <row r="251" spans="1:3">
@@ -3162,7 +3136,7 @@
         <v>7</v>
       </c>
       <c r="C251">
-        <v>1181</v>
+        <v>500000</v>
       </c>
     </row>
     <row r="252" spans="1:3">
@@ -3173,7 +3147,7 @@
         <v>4</v>
       </c>
       <c r="C252">
-        <v>881</v>
+        <v>169000</v>
       </c>
     </row>
     <row r="253" spans="1:3">
@@ -3184,7 +3158,7 @@
         <v>6</v>
       </c>
       <c r="C253">
-        <v>1946</v>
+        <v>482000</v>
       </c>
     </row>
     <row r="254" spans="1:3">
@@ -3195,7 +3169,7 @@
         <v>9</v>
       </c>
       <c r="C254">
-        <v>1337</v>
+        <v>721000</v>
       </c>
     </row>
     <row r="255" spans="1:3">
@@ -3206,7 +3180,7 @@
         <v>9</v>
       </c>
       <c r="C255">
-        <v>1047</v>
+        <v>903000</v>
       </c>
     </row>
     <row r="256" spans="1:3">
@@ -3217,7 +3191,7 @@
         <v>4</v>
       </c>
       <c r="C256">
-        <v>615</v>
+        <v>65000</v>
       </c>
     </row>
     <row r="257" spans="1:3">
@@ -3228,7 +3202,7 @@
         <v>7</v>
       </c>
       <c r="C257">
-        <v>719</v>
+        <v>492000</v>
       </c>
     </row>
     <row r="258" spans="1:3">
@@ -3239,7 +3213,7 @@
         <v>7</v>
       </c>
       <c r="C258">
-        <v>927</v>
+        <v>427000</v>
       </c>
     </row>
     <row r="259" spans="1:3">
@@ -3250,7 +3224,7 @@
         <v>8</v>
       </c>
       <c r="C259">
-        <v>449</v>
+        <v>23000</v>
       </c>
     </row>
     <row r="260" spans="1:3">
@@ -3261,7 +3235,7 @@
         <v>5</v>
       </c>
       <c r="C260">
-        <v>55</v>
+        <v>83000</v>
       </c>
     </row>
     <row r="261" spans="1:3">
@@ -3272,7 +3246,7 @@
         <v>4</v>
       </c>
       <c r="C261">
-        <v>500</v>
+        <v>99000</v>
       </c>
     </row>
     <row r="262" spans="1:3">
@@ -3283,7 +3257,7 @@
         <v>7</v>
       </c>
       <c r="C262">
-        <v>1402</v>
+        <v>274000</v>
       </c>
     </row>
     <row r="263" spans="1:3">
@@ -3294,7 +3268,7 @@
         <v>9</v>
       </c>
       <c r="C263">
-        <v>1006</v>
+        <v>2696000</v>
       </c>
     </row>
     <row r="264" spans="1:3">
@@ -3305,7 +3279,7 @@
         <v>5</v>
       </c>
       <c r="C264">
-        <v>814</v>
+        <v>134000</v>
       </c>
     </row>
     <row r="265" spans="1:3">
@@ -3316,7 +3290,7 @@
         <v>5</v>
       </c>
       <c r="C265">
-        <v>503</v>
+        <v>55000</v>
       </c>
     </row>
     <row r="266" spans="1:3">
@@ -3327,7 +3301,7 @@
         <v>6</v>
       </c>
       <c r="C266">
-        <v>693</v>
+        <v>256000</v>
       </c>
     </row>
     <row r="267" spans="1:3">
@@ -3338,7 +3312,7 @@
         <v>7</v>
       </c>
       <c r="C267">
-        <v>806</v>
+        <v>267000</v>
       </c>
     </row>
     <row r="268" spans="1:3">
@@ -3349,7 +3323,7 @@
         <v>4</v>
       </c>
       <c r="C268">
-        <v>974</v>
+        <v>121000</v>
       </c>
     </row>
     <row r="269" spans="1:3">
@@ -3360,7 +3334,7 @@
         <v>7</v>
       </c>
       <c r="C269">
-        <v>775</v>
+        <v>553000</v>
       </c>
     </row>
     <row r="270" spans="1:3">
@@ -3371,7 +3345,7 @@
         <v>5</v>
       </c>
       <c r="C270">
-        <v>74</v>
+        <v>83000</v>
       </c>
     </row>
     <row r="271" spans="1:3">
@@ -3382,7 +3356,7 @@
         <v>9</v>
       </c>
       <c r="C271">
-        <v>547</v>
+        <v>808000</v>
       </c>
     </row>
     <row r="272" spans="1:3">
@@ -3393,7 +3367,7 @@
         <v>8</v>
       </c>
       <c r="C272">
-        <v>1026</v>
+        <v>66000</v>
       </c>
     </row>
     <row r="273" spans="1:3">
@@ -3404,7 +3378,7 @@
         <v>4</v>
       </c>
       <c r="C273">
-        <v>1952</v>
+        <v>256000</v>
       </c>
     </row>
     <row r="274" spans="1:3">
@@ -3415,7 +3389,7 @@
         <v>9</v>
       </c>
       <c r="C274">
-        <v>825</v>
+        <v>2754000</v>
       </c>
     </row>
     <row r="275" spans="1:3">
@@ -3426,7 +3400,7 @@
         <v>8</v>
       </c>
       <c r="C275">
-        <v>845</v>
+        <v>22000</v>
       </c>
     </row>
     <row r="276" spans="1:3">
@@ -3437,7 +3411,7 @@
         <v>4</v>
       </c>
       <c r="C276">
-        <v>233</v>
+        <v>62000</v>
       </c>
     </row>
     <row r="277" spans="1:3">
@@ -3448,7 +3422,7 @@
         <v>6</v>
       </c>
       <c r="C277">
-        <v>1044</v>
+        <v>373000</v>
       </c>
     </row>
     <row r="278" spans="1:3">
@@ -3459,7 +3433,7 @@
         <v>8</v>
       </c>
       <c r="C278">
-        <v>1184</v>
+        <v>79000</v>
       </c>
     </row>
     <row r="279" spans="1:3">
@@ -3470,7 +3444,7 @@
         <v>7</v>
       </c>
       <c r="C279">
-        <v>797</v>
+        <v>95000</v>
       </c>
     </row>
     <row r="280" spans="1:3">
@@ -3481,7 +3455,7 @@
         <v>8</v>
       </c>
       <c r="C280">
-        <v>655</v>
+        <v>21000</v>
       </c>
     </row>
     <row r="281" spans="1:3">
@@ -3492,7 +3466,7 @@
         <v>5</v>
       </c>
       <c r="C281">
-        <v>1338</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="282" spans="1:3">
@@ -3503,7 +3477,7 @@
         <v>5</v>
       </c>
       <c r="C282">
-        <v>573</v>
+        <v>62000</v>
       </c>
     </row>
     <row r="283" spans="1:3">
@@ -3514,7 +3488,7 @@
         <v>7</v>
       </c>
       <c r="C283">
-        <v>339</v>
+        <v>496000</v>
       </c>
     </row>
     <row r="284" spans="1:3">
@@ -3525,7 +3499,7 @@
         <v>8</v>
       </c>
       <c r="C284">
-        <v>1506</v>
+        <v>72000</v>
       </c>
     </row>
     <row r="285" spans="1:3">
@@ -3536,7 +3510,7 @@
         <v>7</v>
       </c>
       <c r="C285">
-        <v>1545</v>
+        <v>572000</v>
       </c>
     </row>
     <row r="286" spans="1:3">
@@ -3547,7 +3521,7 @@
         <v>8</v>
       </c>
       <c r="C286">
-        <v>217</v>
+        <v>37000</v>
       </c>
     </row>
     <row r="287" spans="1:3">
@@ -3558,7 +3532,7 @@
         <v>9</v>
       </c>
       <c r="C287">
-        <v>1548</v>
+        <v>2142000</v>
       </c>
     </row>
     <row r="288" spans="1:3">
@@ -3569,7 +3543,7 @@
         <v>9</v>
       </c>
       <c r="C288">
-        <v>1430</v>
+        <v>740000</v>
       </c>
     </row>
     <row r="289" spans="1:3">
@@ -3580,7 +3554,7 @@
         <v>6</v>
       </c>
       <c r="C289">
-        <v>728</v>
+        <v>124000</v>
       </c>
     </row>
     <row r="290" spans="1:3">
@@ -3591,7 +3565,7 @@
         <v>3</v>
       </c>
       <c r="C290">
-        <v>840</v>
+        <v>127000</v>
       </c>
     </row>
     <row r="291" spans="1:3">
@@ -3602,7 +3576,7 @@
         <v>5</v>
       </c>
       <c r="C291">
-        <v>1798</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="292" spans="1:3">
@@ -3613,7 +3587,7 @@
         <v>7</v>
       </c>
       <c r="C292">
-        <v>1414</v>
+        <v>479000</v>
       </c>
     </row>
     <row r="293" spans="1:3">
@@ -3624,7 +3598,7 @@
         <v>6</v>
       </c>
       <c r="C293">
-        <v>228</v>
+        <v>175000</v>
       </c>
     </row>
     <row r="294" spans="1:3">
@@ -3635,7 +3609,7 @@
         <v>7</v>
       </c>
       <c r="C294">
-        <v>196</v>
+        <v>545000</v>
       </c>
     </row>
     <row r="295" spans="1:3">
@@ -3646,7 +3620,7 @@
         <v>9</v>
       </c>
       <c r="C295">
-        <v>1559</v>
+        <v>1668000</v>
       </c>
     </row>
     <row r="296" spans="1:3">
@@ -3657,7 +3631,7 @@
         <v>6</v>
       </c>
       <c r="C296">
-        <v>1563</v>
+        <v>256000</v>
       </c>
     </row>
     <row r="297" spans="1:3">
@@ -3668,7 +3642,7 @@
         <v>9</v>
       </c>
       <c r="C297">
-        <v>1315</v>
+        <v>2776000</v>
       </c>
     </row>
     <row r="298" spans="1:3">
@@ -3679,7 +3653,7 @@
         <v>7</v>
       </c>
       <c r="C298">
-        <v>1741</v>
+        <v>757000</v>
       </c>
     </row>
     <row r="299" spans="1:3">
@@ -3690,7 +3664,7 @@
         <v>3</v>
       </c>
       <c r="C299">
-        <v>356</v>
+        <v>154000</v>
       </c>
     </row>
     <row r="300" spans="1:3">
@@ -3701,7 +3675,7 @@
         <v>9</v>
       </c>
       <c r="C300">
-        <v>1022</v>
+        <v>1134000</v>
       </c>
     </row>
     <row r="301" spans="1:3">
@@ -3712,7 +3686,7 @@
         <v>3</v>
       </c>
       <c r="C301">
-        <v>1168</v>
+        <v>78000</v>
       </c>
     </row>
     <row r="302" spans="1:3">
@@ -3723,7 +3697,7 @@
         <v>3</v>
       </c>
       <c r="C302">
-        <v>1251</v>
+        <v>105000</v>
       </c>
     </row>
     <row r="303" spans="1:3">
@@ -3734,7 +3708,7 @@
         <v>7</v>
       </c>
       <c r="C303">
-        <v>225</v>
+        <v>302000</v>
       </c>
     </row>
     <row r="304" spans="1:3">
@@ -3745,7 +3719,7 @@
         <v>7</v>
       </c>
       <c r="C304">
-        <v>1951</v>
+        <v>139000</v>
       </c>
     </row>
     <row r="305" spans="1:3">
@@ -3756,7 +3730,7 @@
         <v>8</v>
       </c>
       <c r="C305">
-        <v>1941</v>
+        <v>79000</v>
       </c>
     </row>
     <row r="306" spans="1:3">
@@ -3767,7 +3741,7 @@
         <v>8</v>
       </c>
       <c r="C306">
-        <v>1905</v>
+        <v>17000</v>
       </c>
     </row>
     <row r="307" spans="1:3">
@@ -3778,7 +3752,7 @@
         <v>4</v>
       </c>
       <c r="C307">
-        <v>1917</v>
+        <v>241000</v>
       </c>
     </row>
     <row r="308" spans="1:3">
@@ -3789,7 +3763,7 @@
         <v>8</v>
       </c>
       <c r="C308">
-        <v>661</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="309" spans="1:3">
@@ -3800,7 +3774,7 @@
         <v>7</v>
       </c>
       <c r="C309">
-        <v>1994</v>
+        <v>138000</v>
       </c>
     </row>
     <row r="310" spans="1:3">
@@ -3811,7 +3785,7 @@
         <v>6</v>
       </c>
       <c r="C310">
-        <v>1822</v>
+        <v>65000</v>
       </c>
     </row>
     <row r="311" spans="1:3">
@@ -3822,7 +3796,7 @@
         <v>5</v>
       </c>
       <c r="C311">
-        <v>1651</v>
+        <v>142000</v>
       </c>
     </row>
     <row r="312" spans="1:3">
@@ -3833,7 +3807,7 @@
         <v>9</v>
       </c>
       <c r="C312">
-        <v>827</v>
+        <v>2559000</v>
       </c>
     </row>
     <row r="313" spans="1:3">
@@ -3844,7 +3818,7 @@
         <v>5</v>
       </c>
       <c r="C313">
-        <v>951</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="314" spans="1:3">
@@ -3855,7 +3829,7 @@
         <v>4</v>
       </c>
       <c r="C314">
-        <v>745</v>
+        <v>64000</v>
       </c>
     </row>
     <row r="315" spans="1:3">
@@ -3866,7 +3840,7 @@
         <v>4</v>
       </c>
       <c r="C315">
-        <v>1390</v>
+        <v>295000</v>
       </c>
     </row>
     <row r="316" spans="1:3">
@@ -3877,7 +3851,7 @@
         <v>8</v>
       </c>
       <c r="C316">
-        <v>1540</v>
+        <v>75000</v>
       </c>
     </row>
     <row r="317" spans="1:3">
@@ -3888,7 +3862,7 @@
         <v>4</v>
       </c>
       <c r="C317">
-        <v>1194</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="318" spans="1:3">
@@ -3899,7 +3873,7 @@
         <v>4</v>
       </c>
       <c r="C318">
-        <v>1279</v>
+        <v>267000</v>
       </c>
     </row>
     <row r="319" spans="1:3">
@@ -3910,7 +3884,7 @@
         <v>7</v>
       </c>
       <c r="C319">
-        <v>27</v>
+        <v>270000</v>
       </c>
     </row>
     <row r="320" spans="1:3">
@@ -3921,7 +3895,7 @@
         <v>3</v>
       </c>
       <c r="C320">
-        <v>1325</v>
+        <v>47000</v>
       </c>
     </row>
     <row r="321" spans="1:3">
@@ -3932,7 +3906,7 @@
         <v>7</v>
       </c>
       <c r="C321">
-        <v>1879</v>
+        <v>689000</v>
       </c>
     </row>
     <row r="322" spans="1:3">
@@ -3943,7 +3917,7 @@
         <v>4</v>
       </c>
       <c r="C322">
-        <v>117</v>
+        <v>67000</v>
       </c>
     </row>
     <row r="323" spans="1:3">
@@ -3954,7 +3928,7 @@
         <v>4</v>
       </c>
       <c r="C323">
-        <v>296</v>
+        <v>222000</v>
       </c>
     </row>
     <row r="324" spans="1:3">
@@ -3965,7 +3939,7 @@
         <v>8</v>
       </c>
       <c r="C324">
-        <v>564</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="325" spans="1:3">
@@ -3976,7 +3950,7 @@
         <v>5</v>
       </c>
       <c r="C325">
-        <v>649</v>
+        <v>123000</v>
       </c>
     </row>
     <row r="326" spans="1:3">
@@ -3987,7 +3961,7 @@
         <v>8</v>
       </c>
       <c r="C326">
-        <v>903</v>
+        <v>25000</v>
       </c>
     </row>
     <row r="327" spans="1:3">
@@ -3998,7 +3972,7 @@
         <v>6</v>
       </c>
       <c r="C327">
-        <v>221</v>
+        <v>495000</v>
       </c>
     </row>
     <row r="328" spans="1:3">
@@ -4009,7 +3983,7 @@
         <v>5</v>
       </c>
       <c r="C328">
-        <v>1546</v>
+        <v>83000</v>
       </c>
     </row>
     <row r="329" spans="1:3">
@@ -4020,7 +3994,7 @@
         <v>5</v>
       </c>
       <c r="C329">
-        <v>1263</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="330" spans="1:3">
@@ -4031,7 +4005,7 @@
         <v>4</v>
       </c>
       <c r="C330">
-        <v>673</v>
+        <v>208000</v>
       </c>
     </row>
     <row r="331" spans="1:3">
@@ -4042,7 +4016,7 @@
         <v>7</v>
       </c>
       <c r="C331">
-        <v>1609</v>
+        <v>163000</v>
       </c>
     </row>
     <row r="332" spans="1:3">
@@ -4053,7 +4027,7 @@
         <v>8</v>
       </c>
       <c r="C332">
-        <v>1051</v>
+        <v>63000</v>
       </c>
     </row>
     <row r="333" spans="1:3">
@@ -4064,7 +4038,7 @@
         <v>7</v>
       </c>
       <c r="C333">
-        <v>885</v>
+        <v>753000</v>
       </c>
     </row>
     <row r="334" spans="1:3">
@@ -4075,7 +4049,7 @@
         <v>8</v>
       </c>
       <c r="C334">
-        <v>973</v>
+        <v>76000</v>
       </c>
     </row>
     <row r="335" spans="1:3">
@@ -4086,7 +4060,7 @@
         <v>9</v>
       </c>
       <c r="C335">
-        <v>876</v>
+        <v>1795000</v>
       </c>
     </row>
     <row r="336" spans="1:3">
@@ -4097,7 +4071,7 @@
         <v>5</v>
       </c>
       <c r="C336">
-        <v>516</v>
+        <v>86000</v>
       </c>
     </row>
     <row r="337" spans="1:3">
@@ -4108,7 +4082,7 @@
         <v>7</v>
       </c>
       <c r="C337">
-        <v>244</v>
+        <v>289000</v>
       </c>
     </row>
     <row r="338" spans="1:3">
@@ -4119,7 +4093,7 @@
         <v>4</v>
       </c>
       <c r="C338">
-        <v>721</v>
+        <v>221000</v>
       </c>
     </row>
     <row r="339" spans="1:3">
@@ -4130,7 +4104,7 @@
         <v>5</v>
       </c>
       <c r="C339">
-        <v>1241</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="340" spans="1:3">
@@ -4141,7 +4115,7 @@
         <v>7</v>
       </c>
       <c r="C340">
-        <v>254</v>
+        <v>324000</v>
       </c>
     </row>
     <row r="341" spans="1:3">
@@ -4152,7 +4126,7 @@
         <v>6</v>
       </c>
       <c r="C341">
-        <v>1765</v>
+        <v>175000</v>
       </c>
     </row>
     <row r="342" spans="1:3">
@@ -4163,7 +4137,7 @@
         <v>3</v>
       </c>
       <c r="C342">
-        <v>257</v>
+        <v>131000</v>
       </c>
     </row>
     <row r="343" spans="1:3">
@@ -4174,7 +4148,7 @@
         <v>9</v>
       </c>
       <c r="C343">
-        <v>141</v>
+        <v>1036000</v>
       </c>
     </row>
     <row r="344" spans="1:3">
@@ -4185,7 +4159,7 @@
         <v>9</v>
       </c>
       <c r="C344">
-        <v>1504</v>
+        <v>1728000</v>
       </c>
     </row>
     <row r="345" spans="1:3">
@@ -4196,7 +4170,7 @@
         <v>8</v>
       </c>
       <c r="C345">
-        <v>343</v>
+        <v>68000</v>
       </c>
     </row>
     <row r="346" spans="1:3">
@@ -4207,7 +4181,7 @@
         <v>9</v>
       </c>
       <c r="C346">
-        <v>553</v>
+        <v>1795000</v>
       </c>
     </row>
     <row r="347" spans="1:3">
@@ -4218,7 +4192,7 @@
         <v>6</v>
       </c>
       <c r="C347">
-        <v>37</v>
+        <v>424000</v>
       </c>
     </row>
     <row r="348" spans="1:3">
@@ -4229,7 +4203,7 @@
         <v>3</v>
       </c>
       <c r="C348">
-        <v>1816</v>
+        <v>48000</v>
       </c>
     </row>
     <row r="349" spans="1:3">
@@ -4240,7 +4214,7 @@
         <v>7</v>
       </c>
       <c r="C349">
-        <v>442</v>
+        <v>89000</v>
       </c>
     </row>
     <row r="350" spans="1:3">
@@ -4251,7 +4225,7 @@
         <v>9</v>
       </c>
       <c r="C350">
-        <v>1312</v>
+        <v>2377000</v>
       </c>
     </row>
     <row r="351" spans="1:3">
@@ -4262,7 +4236,7 @@
         <v>6</v>
       </c>
       <c r="C351">
-        <v>1130</v>
+        <v>358000</v>
       </c>
     </row>
     <row r="352" spans="1:3">
@@ -4273,7 +4247,7 @@
         <v>6</v>
       </c>
       <c r="C352">
-        <v>976</v>
+        <v>328000</v>
       </c>
     </row>
     <row r="353" spans="1:3">
@@ -4284,7 +4258,7 @@
         <v>8</v>
       </c>
       <c r="C353">
-        <v>187</v>
+        <v>22000</v>
       </c>
     </row>
     <row r="354" spans="1:3">
@@ -4295,7 +4269,7 @@
         <v>9</v>
       </c>
       <c r="C354">
-        <v>1599</v>
+        <v>800000</v>
       </c>
     </row>
     <row r="355" spans="1:3">
@@ -4306,7 +4280,7 @@
         <v>4</v>
       </c>
       <c r="C355">
-        <v>1435</v>
+        <v>187000</v>
       </c>
     </row>
     <row r="356" spans="1:3">
@@ -4317,7 +4291,7 @@
         <v>7</v>
       </c>
       <c r="C356">
-        <v>596</v>
+        <v>298000</v>
       </c>
     </row>
     <row r="357" spans="1:3">
@@ -4328,7 +4302,7 @@
         <v>6</v>
       </c>
       <c r="C357">
-        <v>1046</v>
+        <v>299000</v>
       </c>
     </row>
     <row r="358" spans="1:3">
@@ -4339,7 +4313,7 @@
         <v>7</v>
       </c>
       <c r="C358">
-        <v>801</v>
+        <v>351000</v>
       </c>
     </row>
     <row r="359" spans="1:3">
@@ -4350,7 +4324,7 @@
         <v>7</v>
       </c>
       <c r="C359">
-        <v>383</v>
+        <v>215000</v>
       </c>
     </row>
     <row r="360" spans="1:3">
@@ -4361,7 +4335,7 @@
         <v>5</v>
       </c>
       <c r="C360">
-        <v>313</v>
+        <v>109000</v>
       </c>
     </row>
     <row r="361" spans="1:3">
@@ -4372,7 +4346,7 @@
         <v>7</v>
       </c>
       <c r="C361">
-        <v>688</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="362" spans="1:3">
@@ -4383,7 +4357,7 @@
         <v>7</v>
       </c>
       <c r="C362">
-        <v>624</v>
+        <v>330000</v>
       </c>
     </row>
     <row r="363" spans="1:3">
@@ -4394,7 +4368,7 @@
         <v>6</v>
       </c>
       <c r="C363">
-        <v>420</v>
+        <v>229000</v>
       </c>
     </row>
     <row r="364" spans="1:3">
@@ -4405,7 +4379,7 @@
         <v>9</v>
       </c>
       <c r="C364">
-        <v>826</v>
+        <v>1667000</v>
       </c>
     </row>
     <row r="365" spans="1:3">
@@ -4416,7 +4390,7 @@
         <v>3</v>
       </c>
       <c r="C365">
-        <v>797</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="366" spans="1:3">
@@ -4427,7 +4401,7 @@
         <v>3</v>
       </c>
       <c r="C366">
-        <v>1364</v>
+        <v>142000</v>
       </c>
     </row>
     <row r="367" spans="1:3">
@@ -4438,7 +4412,7 @@
         <v>6</v>
       </c>
       <c r="C367">
-        <v>735</v>
+        <v>466000</v>
       </c>
     </row>
     <row r="368" spans="1:3">
@@ -4449,7 +4423,7 @@
         <v>6</v>
       </c>
       <c r="C368">
-        <v>847</v>
+        <v>318000</v>
       </c>
     </row>
     <row r="369" spans="1:3">
@@ -4460,7 +4434,7 @@
         <v>3</v>
       </c>
       <c r="C369">
-        <v>303</v>
+        <v>107000</v>
       </c>
     </row>
     <row r="370" spans="1:3">
@@ -4471,7 +4445,7 @@
         <v>7</v>
       </c>
       <c r="C370">
-        <v>1585</v>
+        <v>706000</v>
       </c>
     </row>
     <row r="371" spans="1:3">
@@ -4482,7 +4456,7 @@
         <v>4</v>
       </c>
       <c r="C371">
-        <v>580</v>
+        <v>256000</v>
       </c>
     </row>
     <row r="372" spans="1:3">
@@ -4493,7 +4467,7 @@
         <v>5</v>
       </c>
       <c r="C372">
-        <v>359</v>
+        <v>22000</v>
       </c>
     </row>
     <row r="373" spans="1:3">
@@ -4504,7 +4478,7 @@
         <v>5</v>
       </c>
       <c r="C373">
-        <v>437</v>
+        <v>96000</v>
       </c>
     </row>
     <row r="374" spans="1:3">
@@ -4515,7 +4489,7 @@
         <v>4</v>
       </c>
       <c r="C374">
-        <v>1040</v>
+        <v>288000</v>
       </c>
     </row>
     <row r="375" spans="1:3">
@@ -4526,7 +4500,7 @@
         <v>3</v>
       </c>
       <c r="C375">
-        <v>958</v>
+        <v>199000</v>
       </c>
     </row>
     <row r="376" spans="1:3">
@@ -4537,7 +4511,7 @@
         <v>7</v>
       </c>
       <c r="C376">
-        <v>334</v>
+        <v>186000</v>
       </c>
     </row>
     <row r="377" spans="1:3">
@@ -4548,7 +4522,7 @@
         <v>7</v>
       </c>
       <c r="C377">
-        <v>167</v>
+        <v>217000</v>
       </c>
     </row>
     <row r="378" spans="1:3">
@@ -4559,7 +4533,7 @@
         <v>8</v>
       </c>
       <c r="C378">
-        <v>920</v>
+        <v>43000</v>
       </c>
     </row>
     <row r="379" spans="1:3">
@@ -4570,7 +4544,7 @@
         <v>8</v>
       </c>
       <c r="C379">
-        <v>1367</v>
+        <v>24000</v>
       </c>
     </row>
     <row r="380" spans="1:3">
@@ -4581,7 +4555,7 @@
         <v>3</v>
       </c>
       <c r="C380">
-        <v>1984</v>
+        <v>57000</v>
       </c>
     </row>
     <row r="381" spans="1:3">
@@ -4592,7 +4566,7 @@
         <v>5</v>
       </c>
       <c r="C381">
-        <v>500</v>
+        <v>59000</v>
       </c>
     </row>
     <row r="382" spans="1:3">
@@ -4603,7 +4577,7 @@
         <v>5</v>
       </c>
       <c r="C382">
-        <v>175</v>
+        <v>89000</v>
       </c>
     </row>
     <row r="383" spans="1:3">
@@ -4614,7 +4588,7 @@
         <v>7</v>
       </c>
       <c r="C383">
-        <v>1375</v>
+        <v>368000</v>
       </c>
     </row>
     <row r="384" spans="1:3">
@@ -4625,7 +4599,7 @@
         <v>7</v>
       </c>
       <c r="C384">
-        <v>161</v>
+        <v>699000</v>
       </c>
     </row>
     <row r="385" spans="1:3">
@@ -4636,7 +4610,7 @@
         <v>8</v>
       </c>
       <c r="C385">
-        <v>1839</v>
+        <v>36000</v>
       </c>
     </row>
     <row r="386" spans="1:3">
@@ -4647,7 +4621,7 @@
         <v>6</v>
       </c>
       <c r="C386">
-        <v>829</v>
+        <v>407000</v>
       </c>
     </row>
     <row r="387" spans="1:3">
@@ -4658,7 +4632,7 @@
         <v>4</v>
       </c>
       <c r="C387">
-        <v>1063</v>
+        <v>137000</v>
       </c>
     </row>
     <row r="388" spans="1:3">
@@ -4669,7 +4643,7 @@
         <v>8</v>
       </c>
       <c r="C388">
-        <v>828</v>
+        <v>36000</v>
       </c>
     </row>
     <row r="389" spans="1:3">
@@ -4680,7 +4654,7 @@
         <v>5</v>
       </c>
       <c r="C389">
-        <v>901</v>
+        <v>87000</v>
       </c>
     </row>
     <row r="390" spans="1:3">
@@ -4691,7 +4665,7 @@
         <v>6</v>
       </c>
       <c r="C390">
-        <v>46</v>
+        <v>298000</v>
       </c>
     </row>
     <row r="391" spans="1:3">
@@ -4702,7 +4676,7 @@
         <v>5</v>
       </c>
       <c r="C391">
-        <v>208</v>
+        <v>145000</v>
       </c>
     </row>
     <row r="392" spans="1:3">
@@ -4713,7 +4687,7 @@
         <v>6</v>
       </c>
       <c r="C392">
-        <v>95</v>
+        <v>168000</v>
       </c>
     </row>
     <row r="393" spans="1:3">
@@ -4724,7 +4698,7 @@
         <v>5</v>
       </c>
       <c r="C393">
-        <v>1008</v>
+        <v>33000</v>
       </c>
     </row>
     <row r="394" spans="1:3">
@@ -4735,7 +4709,7 @@
         <v>5</v>
       </c>
       <c r="C394">
-        <v>1820</v>
+        <v>43000</v>
       </c>
     </row>
     <row r="395" spans="1:3">
@@ -4746,7 +4720,7 @@
         <v>9</v>
       </c>
       <c r="C395">
-        <v>462</v>
+        <v>2234000</v>
       </c>
     </row>
     <row r="396" spans="1:3">
@@ -4757,7 +4731,7 @@
         <v>5</v>
       </c>
       <c r="C396">
-        <v>1073</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="397" spans="1:3">
@@ -4768,7 +4742,7 @@
         <v>3</v>
       </c>
       <c r="C397">
-        <v>1666</v>
+        <v>41000</v>
       </c>
     </row>
     <row r="398" spans="1:3">
@@ -4779,7 +4753,7 @@
         <v>4</v>
       </c>
       <c r="C398">
-        <v>1666</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="399" spans="1:3">
@@ -4790,7 +4764,7 @@
         <v>4</v>
       </c>
       <c r="C399">
-        <v>1229</v>
+        <v>135000</v>
       </c>
     </row>
     <row r="400" spans="1:3">
@@ -4801,7 +4775,7 @@
         <v>9</v>
       </c>
       <c r="C400">
-        <v>54</v>
+        <v>1035000</v>
       </c>
     </row>
     <row r="401" spans="1:3">
@@ -4812,7 +4786,7 @@
         <v>3</v>
       </c>
       <c r="C401">
-        <v>834</v>
+        <v>193000</v>
       </c>
     </row>
     <row r="402" spans="1:3">
@@ -4823,7 +4797,7 @@
         <v>3</v>
       </c>
       <c r="C402">
-        <v>1728</v>
+        <v>97000</v>
       </c>
     </row>
     <row r="403" spans="1:3">
@@ -4834,7 +4808,7 @@
         <v>8</v>
       </c>
       <c r="C403">
-        <v>187</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="404" spans="1:3">
@@ -4845,7 +4819,7 @@
         <v>4</v>
       </c>
       <c r="C404">
-        <v>1328</v>
+        <v>239000</v>
       </c>
     </row>
     <row r="405" spans="1:3">
@@ -4856,7 +4830,7 @@
         <v>6</v>
       </c>
       <c r="C405">
-        <v>1627</v>
+        <v>266000</v>
       </c>
     </row>
     <row r="406" spans="1:3">
@@ -4867,7 +4841,7 @@
         <v>5</v>
       </c>
       <c r="C406">
-        <v>1392</v>
+        <v>129000</v>
       </c>
     </row>
     <row r="407" spans="1:3">
@@ -4878,7 +4852,7 @@
         <v>7</v>
       </c>
       <c r="C407">
-        <v>170</v>
+        <v>654000</v>
       </c>
     </row>
     <row r="408" spans="1:3">
@@ -4889,7 +4863,7 @@
         <v>6</v>
       </c>
       <c r="C408">
-        <v>1934</v>
+        <v>44000</v>
       </c>
     </row>
     <row r="409" spans="1:3">
@@ -4900,7 +4874,7 @@
         <v>3</v>
       </c>
       <c r="C409">
-        <v>288</v>
+        <v>58000</v>
       </c>
     </row>
     <row r="410" spans="1:3">
@@ -4911,7 +4885,7 @@
         <v>8</v>
       </c>
       <c r="C410">
-        <v>231</v>
+        <v>19000</v>
       </c>
     </row>
     <row r="411" spans="1:3">
@@ -4922,7 +4896,7 @@
         <v>5</v>
       </c>
       <c r="C411">
-        <v>711</v>
+        <v>58000</v>
       </c>
     </row>
     <row r="412" spans="1:3">
@@ -4933,7 +4907,7 @@
         <v>8</v>
       </c>
       <c r="C412">
-        <v>1311</v>
+        <v>79000</v>
       </c>
     </row>
     <row r="413" spans="1:3">
@@ -4944,7 +4918,7 @@
         <v>7</v>
       </c>
       <c r="C413">
-        <v>392</v>
+        <v>116000</v>
       </c>
     </row>
     <row r="414" spans="1:3">
@@ -4955,7 +4929,7 @@
         <v>8</v>
       </c>
       <c r="C414">
-        <v>1879</v>
+        <v>57000</v>
       </c>
     </row>
     <row r="415" spans="1:3">
@@ -4966,7 +4940,7 @@
         <v>9</v>
       </c>
       <c r="C415">
-        <v>1561</v>
+        <v>2885000</v>
       </c>
     </row>
     <row r="416" spans="1:3">
@@ -4977,7 +4951,7 @@
         <v>6</v>
       </c>
       <c r="C416">
-        <v>1550</v>
+        <v>322000</v>
       </c>
     </row>
     <row r="417" spans="1:3">
@@ -4988,7 +4962,7 @@
         <v>5</v>
       </c>
       <c r="C417">
-        <v>1507</v>
+        <v>57000</v>
       </c>
     </row>
     <row r="418" spans="1:3">
@@ -4999,7 +4973,7 @@
         <v>9</v>
       </c>
       <c r="C418">
-        <v>517</v>
+        <v>2260000</v>
       </c>
     </row>
     <row r="419" spans="1:3">
@@ -5010,7 +4984,7 @@
         <v>5</v>
       </c>
       <c r="C419">
-        <v>1307</v>
+        <v>52000</v>
       </c>
     </row>
     <row r="420" spans="1:3">
@@ -5021,7 +4995,7 @@
         <v>3</v>
       </c>
       <c r="C420">
-        <v>392</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="421" spans="1:3">
@@ -5032,7 +5006,7 @@
         <v>9</v>
       </c>
       <c r="C421">
-        <v>1241</v>
+        <v>1762000</v>
       </c>
     </row>
     <row r="422" spans="1:3">
@@ -5043,7 +5017,7 @@
         <v>4</v>
       </c>
       <c r="C422">
-        <v>1825</v>
+        <v>143000</v>
       </c>
     </row>
     <row r="423" spans="1:3">
@@ -5054,7 +5028,7 @@
         <v>8</v>
       </c>
       <c r="C423">
-        <v>1065</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="424" spans="1:3">
@@ -5065,7 +5039,7 @@
         <v>3</v>
       </c>
       <c r="C424">
-        <v>917</v>
+        <v>121000</v>
       </c>
     </row>
     <row r="425" spans="1:3">
@@ -5076,7 +5050,7 @@
         <v>4</v>
       </c>
       <c r="C425">
-        <v>1313</v>
+        <v>103000</v>
       </c>
     </row>
     <row r="426" spans="1:3">
@@ -5087,7 +5061,7 @@
         <v>8</v>
       </c>
       <c r="C426">
-        <v>1926</v>
+        <v>41000</v>
       </c>
     </row>
     <row r="427" spans="1:3">
@@ -5098,7 +5072,7 @@
         <v>9</v>
       </c>
       <c r="C427">
-        <v>271</v>
+        <v>921000</v>
       </c>
     </row>
     <row r="428" spans="1:3">
@@ -5109,7 +5083,7 @@
         <v>9</v>
       </c>
       <c r="C428">
-        <v>1888</v>
+        <v>1948000</v>
       </c>
     </row>
     <row r="429" spans="1:3">
@@ -5120,7 +5094,7 @@
         <v>7</v>
       </c>
       <c r="C429">
-        <v>37</v>
+        <v>653000</v>
       </c>
     </row>
     <row r="430" spans="1:3">
@@ -5131,7 +5105,7 @@
         <v>8</v>
       </c>
       <c r="C430">
-        <v>749</v>
+        <v>62000</v>
       </c>
     </row>
     <row r="431" spans="1:3">
@@ -5142,7 +5116,7 @@
         <v>7</v>
       </c>
       <c r="C431">
-        <v>1367</v>
+        <v>715000</v>
       </c>
     </row>
     <row r="432" spans="1:3">
@@ -5153,7 +5127,7 @@
         <v>3</v>
       </c>
       <c r="C432">
-        <v>102</v>
+        <v>69000</v>
       </c>
     </row>
     <row r="433" spans="1:3">
@@ -5164,7 +5138,7 @@
         <v>9</v>
       </c>
       <c r="C433">
-        <v>1785</v>
+        <v>1469000</v>
       </c>
     </row>
     <row r="434" spans="1:3">
@@ -5175,7 +5149,7 @@
         <v>7</v>
       </c>
       <c r="C434">
-        <v>1524</v>
+        <v>246000</v>
       </c>
     </row>
     <row r="435" spans="1:3">
@@ -5186,7 +5160,7 @@
         <v>8</v>
       </c>
       <c r="C435">
-        <v>1263</v>
+        <v>32000</v>
       </c>
     </row>
     <row r="436" spans="1:3">
@@ -5197,7 +5171,7 @@
         <v>9</v>
       </c>
       <c r="C436">
-        <v>1195</v>
+        <v>2188000</v>
       </c>
     </row>
     <row r="437" spans="1:3">
@@ -5208,7 +5182,7 @@
         <v>5</v>
       </c>
       <c r="C437">
-        <v>1749</v>
+        <v>26000</v>
       </c>
     </row>
     <row r="438" spans="1:3">
@@ -5219,7 +5193,7 @@
         <v>3</v>
       </c>
       <c r="C438">
-        <v>149</v>
+        <v>75000</v>
       </c>
     </row>
     <row r="439" spans="1:3">
@@ -5230,7 +5204,7 @@
         <v>4</v>
       </c>
       <c r="C439">
-        <v>542</v>
+        <v>238000</v>
       </c>
     </row>
     <row r="440" spans="1:3">
@@ -5241,7 +5215,7 @@
         <v>4</v>
       </c>
       <c r="C440">
-        <v>756</v>
+        <v>286000</v>
       </c>
     </row>
     <row r="441" spans="1:3">
@@ -5252,7 +5226,7 @@
         <v>9</v>
       </c>
       <c r="C441">
-        <v>1906</v>
+        <v>1860000</v>
       </c>
     </row>
     <row r="442" spans="1:3">
@@ -5263,7 +5237,7 @@
         <v>9</v>
       </c>
       <c r="C442">
-        <v>94</v>
+        <v>2186000</v>
       </c>
     </row>
     <row r="443" spans="1:3">
@@ -5274,7 +5248,7 @@
         <v>5</v>
       </c>
       <c r="C443">
-        <v>537</v>
+        <v>83000</v>
       </c>
     </row>
     <row r="444" spans="1:3">
@@ -5285,7 +5259,7 @@
         <v>6</v>
       </c>
       <c r="C444">
-        <v>683</v>
+        <v>176000</v>
       </c>
     </row>
     <row r="445" spans="1:3">
@@ -5296,7 +5270,7 @@
         <v>6</v>
       </c>
       <c r="C445">
-        <v>1615</v>
+        <v>121000</v>
       </c>
     </row>
     <row r="446" spans="1:3">
@@ -5307,7 +5281,7 @@
         <v>5</v>
       </c>
       <c r="C446">
-        <v>219</v>
+        <v>47000</v>
       </c>
     </row>
     <row r="447" spans="1:3">
@@ -5318,7 +5292,7 @@
         <v>4</v>
       </c>
       <c r="C447">
-        <v>1125</v>
+        <v>147000</v>
       </c>
     </row>
     <row r="448" spans="1:3">
@@ -5329,7 +5303,7 @@
         <v>6</v>
       </c>
       <c r="C448">
-        <v>1529</v>
+        <v>486000</v>
       </c>
     </row>
     <row r="449" spans="1:3">
@@ -5340,7 +5314,7 @@
         <v>6</v>
       </c>
       <c r="C449">
-        <v>815</v>
+        <v>59000</v>
       </c>
     </row>
     <row r="450" spans="1:3">
@@ -5351,7 +5325,7 @@
         <v>7</v>
       </c>
       <c r="C450">
-        <v>1064</v>
+        <v>561000</v>
       </c>
     </row>
     <row r="451" spans="1:3">
@@ -5362,7 +5336,7 @@
         <v>9</v>
       </c>
       <c r="C451">
-        <v>1482</v>
+        <v>1411000</v>
       </c>
     </row>
     <row r="452" spans="1:3">
@@ -5373,7 +5347,7 @@
         <v>3</v>
       </c>
       <c r="C452">
-        <v>365</v>
+        <v>81000</v>
       </c>
     </row>
     <row r="453" spans="1:3">
@@ -5384,7 +5358,7 @@
         <v>6</v>
       </c>
       <c r="C453">
-        <v>858</v>
+        <v>458000</v>
       </c>
     </row>
     <row r="454" spans="1:3">
@@ -5395,7 +5369,7 @@
         <v>6</v>
       </c>
       <c r="C454">
-        <v>1347</v>
+        <v>275000</v>
       </c>
     </row>
     <row r="455" spans="1:3">
@@ -5406,7 +5380,7 @@
         <v>6</v>
       </c>
       <c r="C455">
-        <v>756</v>
+        <v>219000</v>
       </c>
     </row>
     <row r="456" spans="1:3">
@@ -5417,7 +5391,7 @@
         <v>6</v>
       </c>
       <c r="C456">
-        <v>1006</v>
+        <v>196000</v>
       </c>
     </row>
     <row r="457" spans="1:3">
@@ -5428,7 +5402,7 @@
         <v>7</v>
       </c>
       <c r="C457">
-        <v>552</v>
+        <v>313000</v>
       </c>
     </row>
     <row r="458" spans="1:3">
@@ -5439,7 +5413,7 @@
         <v>4</v>
       </c>
       <c r="C458">
-        <v>1143</v>
+        <v>107000</v>
       </c>
     </row>
     <row r="459" spans="1:3">
@@ -5450,7 +5424,7 @@
         <v>6</v>
       </c>
       <c r="C459">
-        <v>24</v>
+        <v>52000</v>
       </c>
     </row>
     <row r="460" spans="1:3">
@@ -5461,7 +5435,7 @@
         <v>9</v>
       </c>
       <c r="C460">
-        <v>806</v>
+        <v>1291000</v>
       </c>
     </row>
     <row r="461" spans="1:3">
@@ -5472,7 +5446,7 @@
         <v>5</v>
       </c>
       <c r="C461">
-        <v>1609</v>
+        <v>122000</v>
       </c>
     </row>
     <row r="462" spans="1:3">
@@ -5483,7 +5457,7 @@
         <v>6</v>
       </c>
       <c r="C462">
-        <v>1548</v>
+        <v>208000</v>
       </c>
     </row>
     <row r="463" spans="1:3">
@@ -5494,7 +5468,7 @@
         <v>6</v>
       </c>
       <c r="C463">
-        <v>1736</v>
+        <v>182000</v>
       </c>
     </row>
     <row r="464" spans="1:3">
@@ -5505,7 +5479,7 @@
         <v>4</v>
       </c>
       <c r="C464">
-        <v>134</v>
+        <v>271000</v>
       </c>
     </row>
     <row r="465" spans="1:3">
@@ -5516,7 +5490,7 @@
         <v>3</v>
       </c>
       <c r="C465">
-        <v>1926</v>
+        <v>47000</v>
       </c>
     </row>
     <row r="466" spans="1:3">
@@ -5527,7 +5501,7 @@
         <v>9</v>
       </c>
       <c r="C466">
-        <v>1948</v>
+        <v>1643000</v>
       </c>
     </row>
     <row r="467" spans="1:3">
@@ -5538,7 +5512,7 @@
         <v>7</v>
       </c>
       <c r="C467">
-        <v>1543</v>
+        <v>439000</v>
       </c>
     </row>
     <row r="468" spans="1:3">
@@ -5549,7 +5523,7 @@
         <v>9</v>
       </c>
       <c r="C468">
-        <v>1635</v>
+        <v>2586000</v>
       </c>
     </row>
     <row r="469" spans="1:3">
@@ -5560,7 +5534,7 @@
         <v>4</v>
       </c>
       <c r="C469">
-        <v>881</v>
+        <v>152000</v>
       </c>
     </row>
     <row r="470" spans="1:3">
@@ -5571,7 +5545,7 @@
         <v>5</v>
       </c>
       <c r="C470">
-        <v>110</v>
+        <v>104000</v>
       </c>
     </row>
     <row r="471" spans="1:3">
@@ -5582,7 +5556,7 @@
         <v>9</v>
       </c>
       <c r="C471">
-        <v>49</v>
+        <v>613000</v>
       </c>
     </row>
     <row r="472" spans="1:3">
@@ -5593,7 +5567,7 @@
         <v>6</v>
       </c>
       <c r="C472">
-        <v>1781</v>
+        <v>99000</v>
       </c>
     </row>
     <row r="473" spans="1:3">
@@ -5604,7 +5578,7 @@
         <v>6</v>
       </c>
       <c r="C473">
-        <v>768</v>
+        <v>489000</v>
       </c>
     </row>
     <row r="474" spans="1:3">
@@ -5615,7 +5589,7 @@
         <v>7</v>
       </c>
       <c r="C474">
-        <v>1178</v>
+        <v>347000</v>
       </c>
     </row>
     <row r="475" spans="1:3">
@@ -5626,7 +5600,7 @@
         <v>8</v>
       </c>
       <c r="C475">
-        <v>779</v>
+        <v>32000</v>
       </c>
     </row>
     <row r="476" spans="1:3">
@@ -5637,7 +5611,7 @@
         <v>3</v>
       </c>
       <c r="C476">
-        <v>528</v>
+        <v>178000</v>
       </c>
     </row>
     <row r="477" spans="1:3">
@@ -5648,7 +5622,7 @@
         <v>3</v>
       </c>
       <c r="C477">
-        <v>936</v>
+        <v>97000</v>
       </c>
     </row>
     <row r="478" spans="1:3">
@@ -5659,7 +5633,7 @@
         <v>4</v>
       </c>
       <c r="C478">
-        <v>1641</v>
+        <v>59000</v>
       </c>
     </row>
     <row r="479" spans="1:3">
@@ -5670,7 +5644,7 @@
         <v>3</v>
       </c>
       <c r="C479">
-        <v>1158</v>
+        <v>57000</v>
       </c>
     </row>
     <row r="480" spans="1:3">
@@ -5681,7 +5655,7 @@
         <v>4</v>
       </c>
       <c r="C480">
-        <v>1609</v>
+        <v>202000</v>
       </c>
     </row>
     <row r="481" spans="1:3">
@@ -5692,7 +5666,7 @@
         <v>7</v>
       </c>
       <c r="C481">
-        <v>568</v>
+        <v>524000</v>
       </c>
     </row>
     <row r="482" spans="1:3">
@@ -5703,7 +5677,7 @@
         <v>5</v>
       </c>
       <c r="C482">
-        <v>306</v>
+        <v>108000</v>
       </c>
     </row>
     <row r="483" spans="1:3">
@@ -5714,7 +5688,7 @@
         <v>6</v>
       </c>
       <c r="C483">
-        <v>481</v>
+        <v>413000</v>
       </c>
     </row>
     <row r="484" spans="1:3">
@@ -5725,7 +5699,7 @@
         <v>5</v>
       </c>
       <c r="C484">
-        <v>563</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="485" spans="1:3">
@@ -5736,7 +5710,7 @@
         <v>6</v>
       </c>
       <c r="C485">
-        <v>532</v>
+        <v>263000</v>
       </c>
     </row>
     <row r="486" spans="1:3">
@@ -5747,7 +5721,7 @@
         <v>6</v>
       </c>
       <c r="C486">
-        <v>685</v>
+        <v>350000</v>
       </c>
     </row>
     <row r="487" spans="1:3">
@@ -5758,7 +5732,7 @@
         <v>9</v>
       </c>
       <c r="C487">
-        <v>397</v>
+        <v>2594000</v>
       </c>
     </row>
     <row r="488" spans="1:3">
@@ -5769,7 +5743,7 @@
         <v>7</v>
       </c>
       <c r="C488">
-        <v>313</v>
+        <v>198000</v>
       </c>
     </row>
     <row r="489" spans="1:3">
@@ -5780,7 +5754,7 @@
         <v>9</v>
       </c>
       <c r="C489">
-        <v>560</v>
+        <v>2077000</v>
       </c>
     </row>
     <row r="490" spans="1:3">
@@ -5791,7 +5765,7 @@
         <v>6</v>
       </c>
       <c r="C490">
-        <v>818</v>
+        <v>500000</v>
       </c>
     </row>
     <row r="491" spans="1:3">
@@ -5802,7 +5776,7 @@
         <v>4</v>
       </c>
       <c r="C491">
-        <v>879</v>
+        <v>197000</v>
       </c>
     </row>
     <row r="492" spans="1:3">
@@ -5813,7 +5787,7 @@
         <v>9</v>
       </c>
       <c r="C492">
-        <v>595</v>
+        <v>1278000</v>
       </c>
     </row>
     <row r="493" spans="1:3">
@@ -5824,7 +5798,7 @@
         <v>5</v>
       </c>
       <c r="C493">
-        <v>1919</v>
+        <v>85000</v>
       </c>
     </row>
     <row r="494" spans="1:3">
@@ -5835,7 +5809,7 @@
         <v>5</v>
       </c>
       <c r="C494">
-        <v>300</v>
+        <v>31000</v>
       </c>
     </row>
     <row r="495" spans="1:3">
@@ -5846,7 +5820,7 @@
         <v>8</v>
       </c>
       <c r="C495">
-        <v>693</v>
+        <v>65000</v>
       </c>
     </row>
     <row r="496" spans="1:3">
@@ -5857,7 +5831,7 @@
         <v>8</v>
       </c>
       <c r="C496">
-        <v>1111</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="497" spans="1:3">
@@ -5868,7 +5842,7 @@
         <v>9</v>
       </c>
       <c r="C497">
-        <v>674</v>
+        <v>2629000</v>
       </c>
     </row>
     <row r="498" spans="1:3">
@@ -5879,7 +5853,7 @@
         <v>8</v>
       </c>
       <c r="C498">
-        <v>1944</v>
+        <v>78000</v>
       </c>
     </row>
     <row r="499" spans="1:3">
@@ -5890,7 +5864,7 @@
         <v>7</v>
       </c>
       <c r="C499">
-        <v>783</v>
+        <v>783000</v>
       </c>
     </row>
     <row r="500" spans="1:3">
@@ -5901,7 +5875,7 @@
         <v>5</v>
       </c>
       <c r="C500">
-        <v>1704</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="501" spans="1:3">
@@ -5912,7 +5886,7 @@
         <v>9</v>
       </c>
       <c r="C501">
-        <v>1351</v>
+        <v>1991000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
↩️ Restore original dataset (countries, categories, prices)
</commit_message>
<xml_diff>
--- a/data/products.xlsx
+++ b/data/products.xlsx
@@ -25,33 +25,41 @@
     <t>price</t>
   </si>
   <si>
-    <t>ألعاب</t>
+    <t>Toys</t>
   </si>
   <si>
-    <t>ملابس</t>
+    <t>Clothes</t>
   </si>
   <si>
-    <t>عناية شخصية</t>
+    <t>Perfumes</t>
   </si>
   <si>
-    <t>رياضة</t>
+    <t>Sports</t>
   </si>
   <si>
-    <t>منزل وديكور</t>
+    <t>Home Appliances</t>
   </si>
   <si>
-    <t>كتب</t>
+    <t>Books</t>
   </si>
   <si>
-    <t>إلكترونيات</t>
+    <t>Electronics</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -67,7 +75,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -75,12 +83,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -379,13 +405,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -397,7 +423,7 @@
         <v>3</v>
       </c>
       <c r="C2">
-        <v>193000</v>
+        <v>1351</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -408,7 +434,7 @@
         <v>3</v>
       </c>
       <c r="C3">
-        <v>58000</v>
+        <v>874</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -419,7 +445,7 @@
         <v>3</v>
       </c>
       <c r="C4">
-        <v>36000</v>
+        <v>1686</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -430,7 +456,7 @@
         <v>4</v>
       </c>
       <c r="C5">
-        <v>239000</v>
+        <v>1453</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -441,7 +467,7 @@
         <v>5</v>
       </c>
       <c r="C6">
-        <v>90000</v>
+        <v>1215</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -452,7 +478,7 @@
         <v>3</v>
       </c>
       <c r="C7">
-        <v>92000</v>
+        <v>972</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -463,7 +489,7 @@
         <v>5</v>
       </c>
       <c r="C8">
-        <v>77000</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -474,7 +500,7 @@
         <v>5</v>
       </c>
       <c r="C9">
-        <v>55000</v>
+        <v>62</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -485,7 +511,7 @@
         <v>5</v>
       </c>
       <c r="C10">
-        <v>46000</v>
+        <v>1666</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -496,7 +522,7 @@
         <v>6</v>
       </c>
       <c r="C11">
-        <v>386000</v>
+        <v>1298</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -507,7 +533,7 @@
         <v>6</v>
       </c>
       <c r="C12">
-        <v>419000</v>
+        <v>668</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -518,7 +544,7 @@
         <v>7</v>
       </c>
       <c r="C13">
-        <v>638000</v>
+        <v>1540</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -529,7 +555,7 @@
         <v>8</v>
       </c>
       <c r="C14">
-        <v>21000</v>
+        <v>1694</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -540,7 +566,7 @@
         <v>3</v>
       </c>
       <c r="C15">
-        <v>181000</v>
+        <v>177</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -551,7 +577,7 @@
         <v>9</v>
       </c>
       <c r="C16">
-        <v>2228000</v>
+        <v>346</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -562,7 +588,7 @@
         <v>5</v>
       </c>
       <c r="C17">
-        <v>28000</v>
+        <v>1620</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -573,7 +599,7 @@
         <v>5</v>
       </c>
       <c r="C18">
-        <v>27000</v>
+        <v>960</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -584,7 +610,7 @@
         <v>4</v>
       </c>
       <c r="C19">
-        <v>73000</v>
+        <v>1969</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -595,7 +621,7 @@
         <v>5</v>
       </c>
       <c r="C20">
-        <v>75000</v>
+        <v>1186</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -606,7 +632,7 @@
         <v>7</v>
       </c>
       <c r="C21">
-        <v>318000</v>
+        <v>34</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -617,7 +643,7 @@
         <v>4</v>
       </c>
       <c r="C22">
-        <v>179000</v>
+        <v>179</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -628,7 +654,7 @@
         <v>9</v>
       </c>
       <c r="C23">
-        <v>2965000</v>
+        <v>1308</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -639,7 +665,7 @@
         <v>5</v>
       </c>
       <c r="C24">
-        <v>26000</v>
+        <v>1448</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -650,7 +676,7 @@
         <v>4</v>
       </c>
       <c r="C25">
-        <v>193000</v>
+        <v>863</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -661,7 +687,7 @@
         <v>3</v>
       </c>
       <c r="C26">
-        <v>80000</v>
+        <v>1473</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -672,7 +698,7 @@
         <v>3</v>
       </c>
       <c r="C27">
-        <v>196000</v>
+        <v>139</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -683,7 +709,7 @@
         <v>7</v>
       </c>
       <c r="C28">
-        <v>798000</v>
+        <v>1439</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -694,7 +720,7 @@
         <v>6</v>
       </c>
       <c r="C29">
-        <v>319000</v>
+        <v>1825</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -705,7 +731,7 @@
         <v>9</v>
       </c>
       <c r="C30">
-        <v>2218000</v>
+        <v>1279</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -716,7 +742,7 @@
         <v>8</v>
       </c>
       <c r="C31">
-        <v>38000</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -727,7 +753,7 @@
         <v>3</v>
       </c>
       <c r="C32">
-        <v>144000</v>
+        <v>1847</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -738,7 +764,7 @@
         <v>8</v>
       </c>
       <c r="C33">
-        <v>45000</v>
+        <v>74</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -749,7 +775,7 @@
         <v>4</v>
       </c>
       <c r="C34">
-        <v>257000</v>
+        <v>805</v>
       </c>
     </row>
     <row r="35" spans="1:3">
@@ -760,7 +786,7 @@
         <v>7</v>
       </c>
       <c r="C35">
-        <v>86000</v>
+        <v>372</v>
       </c>
     </row>
     <row r="36" spans="1:3">
@@ -771,7 +797,7 @@
         <v>4</v>
       </c>
       <c r="C36">
-        <v>244000</v>
+        <v>286</v>
       </c>
     </row>
     <row r="37" spans="1:3">
@@ -782,7 +808,7 @@
         <v>4</v>
       </c>
       <c r="C37">
-        <v>256000</v>
+        <v>421</v>
       </c>
     </row>
     <row r="38" spans="1:3">
@@ -793,7 +819,7 @@
         <v>6</v>
       </c>
       <c r="C38">
-        <v>121000</v>
+        <v>635</v>
       </c>
     </row>
     <row r="39" spans="1:3">
@@ -804,7 +830,7 @@
         <v>7</v>
       </c>
       <c r="C39">
-        <v>794000</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="40" spans="1:3">
@@ -815,7 +841,7 @@
         <v>5</v>
       </c>
       <c r="C40">
-        <v>128000</v>
+        <v>339</v>
       </c>
     </row>
     <row r="41" spans="1:3">
@@ -826,7 +852,7 @@
         <v>7</v>
       </c>
       <c r="C41">
-        <v>428000</v>
+        <v>1808</v>
       </c>
     </row>
     <row r="42" spans="1:3">
@@ -837,7 +863,7 @@
         <v>3</v>
       </c>
       <c r="C42">
-        <v>101000</v>
+        <v>1574</v>
       </c>
     </row>
     <row r="43" spans="1:3">
@@ -848,7 +874,7 @@
         <v>7</v>
       </c>
       <c r="C43">
-        <v>239000</v>
+        <v>1957</v>
       </c>
     </row>
     <row r="44" spans="1:3">
@@ -859,7 +885,7 @@
         <v>9</v>
       </c>
       <c r="C44">
-        <v>1381000</v>
+        <v>1673</v>
       </c>
     </row>
     <row r="45" spans="1:3">
@@ -870,7 +896,7 @@
         <v>8</v>
       </c>
       <c r="C45">
-        <v>53000</v>
+        <v>1464</v>
       </c>
     </row>
     <row r="46" spans="1:3">
@@ -881,7 +907,7 @@
         <v>5</v>
       </c>
       <c r="C46">
-        <v>46000</v>
+        <v>124</v>
       </c>
     </row>
     <row r="47" spans="1:3">
@@ -892,7 +918,7 @@
         <v>8</v>
       </c>
       <c r="C47">
-        <v>21000</v>
+        <v>427</v>
       </c>
     </row>
     <row r="48" spans="1:3">
@@ -903,7 +929,7 @@
         <v>9</v>
       </c>
       <c r="C48">
-        <v>2056000</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="49" spans="1:3">
@@ -914,7 +940,7 @@
         <v>3</v>
       </c>
       <c r="C49">
-        <v>54000</v>
+        <v>58</v>
       </c>
     </row>
     <row r="50" spans="1:3">
@@ -925,7 +951,7 @@
         <v>3</v>
       </c>
       <c r="C50">
-        <v>121000</v>
+        <v>312</v>
       </c>
     </row>
     <row r="51" spans="1:3">
@@ -936,7 +962,7 @@
         <v>3</v>
       </c>
       <c r="C51">
-        <v>118000</v>
+        <v>1594</v>
       </c>
     </row>
     <row r="52" spans="1:3">
@@ -947,7 +973,7 @@
         <v>3</v>
       </c>
       <c r="C52">
-        <v>184000</v>
+        <v>536</v>
       </c>
     </row>
     <row r="53" spans="1:3">
@@ -958,7 +984,7 @@
         <v>3</v>
       </c>
       <c r="C53">
-        <v>97000</v>
+        <v>747</v>
       </c>
     </row>
     <row r="54" spans="1:3">
@@ -969,7 +995,7 @@
         <v>6</v>
       </c>
       <c r="C54">
-        <v>453000</v>
+        <v>182</v>
       </c>
     </row>
     <row r="55" spans="1:3">
@@ -980,7 +1006,7 @@
         <v>6</v>
       </c>
       <c r="C55">
-        <v>62000</v>
+        <v>637</v>
       </c>
     </row>
     <row r="56" spans="1:3">
@@ -991,7 +1017,7 @@
         <v>7</v>
       </c>
       <c r="C56">
-        <v>550000</v>
+        <v>207</v>
       </c>
     </row>
     <row r="57" spans="1:3">
@@ -1002,7 +1028,7 @@
         <v>3</v>
       </c>
       <c r="C57">
-        <v>167000</v>
+        <v>73</v>
       </c>
     </row>
     <row r="58" spans="1:3">
@@ -1013,7 +1039,7 @@
         <v>6</v>
       </c>
       <c r="C58">
-        <v>103000</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="59" spans="1:3">
@@ -1024,7 +1050,7 @@
         <v>7</v>
       </c>
       <c r="C59">
-        <v>467000</v>
+        <v>794</v>
       </c>
     </row>
     <row r="60" spans="1:3">
@@ -1035,7 +1061,7 @@
         <v>9</v>
       </c>
       <c r="C60">
-        <v>822000</v>
+        <v>421</v>
       </c>
     </row>
     <row r="61" spans="1:3">
@@ -1046,7 +1072,7 @@
         <v>6</v>
       </c>
       <c r="C61">
-        <v>322000</v>
+        <v>1314</v>
       </c>
     </row>
     <row r="62" spans="1:3">
@@ -1057,7 +1083,7 @@
         <v>8</v>
       </c>
       <c r="C62">
-        <v>47000</v>
+        <v>475</v>
       </c>
     </row>
     <row r="63" spans="1:3">
@@ -1068,7 +1094,7 @@
         <v>9</v>
       </c>
       <c r="C63">
-        <v>1981000</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="64" spans="1:3">
@@ -1079,7 +1105,7 @@
         <v>3</v>
       </c>
       <c r="C64">
-        <v>177000</v>
+        <v>1806</v>
       </c>
     </row>
     <row r="65" spans="1:3">
@@ -1090,7 +1116,7 @@
         <v>6</v>
       </c>
       <c r="C65">
-        <v>138000</v>
+        <v>1624</v>
       </c>
     </row>
     <row r="66" spans="1:3">
@@ -1101,7 +1127,7 @@
         <v>8</v>
       </c>
       <c r="C66">
-        <v>18000</v>
+        <v>1432</v>
       </c>
     </row>
     <row r="67" spans="1:3">
@@ -1112,7 +1138,7 @@
         <v>3</v>
       </c>
       <c r="C67">
-        <v>41000</v>
+        <v>1701</v>
       </c>
     </row>
     <row r="68" spans="1:3">
@@ -1123,7 +1149,7 @@
         <v>9</v>
       </c>
       <c r="C68">
-        <v>1433000</v>
+        <v>1630</v>
       </c>
     </row>
     <row r="69" spans="1:3">
@@ -1134,7 +1160,7 @@
         <v>5</v>
       </c>
       <c r="C69">
-        <v>94000</v>
+        <v>1695</v>
       </c>
     </row>
     <row r="70" spans="1:3">
@@ -1145,7 +1171,7 @@
         <v>3</v>
       </c>
       <c r="C70">
-        <v>50000</v>
+        <v>567</v>
       </c>
     </row>
     <row r="71" spans="1:3">
@@ -1156,7 +1182,7 @@
         <v>3</v>
       </c>
       <c r="C71">
-        <v>89000</v>
+        <v>1508</v>
       </c>
     </row>
     <row r="72" spans="1:3">
@@ -1167,7 +1193,7 @@
         <v>8</v>
       </c>
       <c r="C72">
-        <v>22000</v>
+        <v>334</v>
       </c>
     </row>
     <row r="73" spans="1:3">
@@ -1178,7 +1204,7 @@
         <v>9</v>
       </c>
       <c r="C73">
-        <v>2056000</v>
+        <v>40</v>
       </c>
     </row>
     <row r="74" spans="1:3">
@@ -1189,7 +1215,7 @@
         <v>8</v>
       </c>
       <c r="C74">
-        <v>45000</v>
+        <v>1876</v>
       </c>
     </row>
     <row r="75" spans="1:3">
@@ -1200,7 +1226,7 @@
         <v>5</v>
       </c>
       <c r="C75">
-        <v>136000</v>
+        <v>36</v>
       </c>
     </row>
     <row r="76" spans="1:3">
@@ -1211,7 +1237,7 @@
         <v>4</v>
       </c>
       <c r="C76">
-        <v>212000</v>
+        <v>493</v>
       </c>
     </row>
     <row r="77" spans="1:3">
@@ -1222,7 +1248,7 @@
         <v>6</v>
       </c>
       <c r="C77">
-        <v>467000</v>
+        <v>118</v>
       </c>
     </row>
     <row r="78" spans="1:3">
@@ -1233,7 +1259,7 @@
         <v>9</v>
       </c>
       <c r="C78">
-        <v>1994000</v>
+        <v>187</v>
       </c>
     </row>
     <row r="79" spans="1:3">
@@ -1244,7 +1270,7 @@
         <v>4</v>
       </c>
       <c r="C79">
-        <v>91000</v>
+        <v>716</v>
       </c>
     </row>
     <row r="80" spans="1:3">
@@ -1255,7 +1281,7 @@
         <v>4</v>
       </c>
       <c r="C80">
-        <v>144000</v>
+        <v>440</v>
       </c>
     </row>
     <row r="81" spans="1:3">
@@ -1266,7 +1292,7 @@
         <v>6</v>
       </c>
       <c r="C81">
-        <v>221000</v>
+        <v>174</v>
       </c>
     </row>
     <row r="82" spans="1:3">
@@ -1277,7 +1303,7 @@
         <v>3</v>
       </c>
       <c r="C82">
-        <v>83000</v>
+        <v>734</v>
       </c>
     </row>
     <row r="83" spans="1:3">
@@ -1288,7 +1314,7 @@
         <v>8</v>
       </c>
       <c r="C83">
-        <v>44000</v>
+        <v>1689</v>
       </c>
     </row>
     <row r="84" spans="1:3">
@@ -1299,7 +1325,7 @@
         <v>8</v>
       </c>
       <c r="C84">
-        <v>19000</v>
+        <v>352</v>
       </c>
     </row>
     <row r="85" spans="1:3">
@@ -1310,7 +1336,7 @@
         <v>8</v>
       </c>
       <c r="C85">
-        <v>31000</v>
+        <v>77</v>
       </c>
     </row>
     <row r="86" spans="1:3">
@@ -1321,7 +1347,7 @@
         <v>8</v>
       </c>
       <c r="C86">
-        <v>78000</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="87" spans="1:3">
@@ -1332,7 +1358,7 @@
         <v>6</v>
       </c>
       <c r="C87">
-        <v>413000</v>
+        <v>205</v>
       </c>
     </row>
     <row r="88" spans="1:3">
@@ -1343,7 +1369,7 @@
         <v>6</v>
       </c>
       <c r="C88">
-        <v>165000</v>
+        <v>1636</v>
       </c>
     </row>
     <row r="89" spans="1:3">
@@ -1354,7 +1380,7 @@
         <v>8</v>
       </c>
       <c r="C89">
-        <v>30000</v>
+        <v>1404</v>
       </c>
     </row>
     <row r="90" spans="1:3">
@@ -1365,7 +1391,7 @@
         <v>6</v>
       </c>
       <c r="C90">
-        <v>276000</v>
+        <v>522</v>
       </c>
     </row>
     <row r="91" spans="1:3">
@@ -1376,7 +1402,7 @@
         <v>6</v>
       </c>
       <c r="C91">
-        <v>234000</v>
+        <v>418</v>
       </c>
     </row>
     <row r="92" spans="1:3">
@@ -1387,7 +1413,7 @@
         <v>7</v>
       </c>
       <c r="C92">
-        <v>356000</v>
+        <v>72</v>
       </c>
     </row>
     <row r="93" spans="1:3">
@@ -1398,7 +1424,7 @@
         <v>6</v>
       </c>
       <c r="C93">
-        <v>367000</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="94" spans="1:3">
@@ -1409,7 +1435,7 @@
         <v>8</v>
       </c>
       <c r="C94">
-        <v>38000</v>
+        <v>1949</v>
       </c>
     </row>
     <row r="95" spans="1:3">
@@ -1420,7 +1446,7 @@
         <v>4</v>
       </c>
       <c r="C95">
-        <v>225000</v>
+        <v>594</v>
       </c>
     </row>
     <row r="96" spans="1:3">
@@ -1431,7 +1457,7 @@
         <v>5</v>
       </c>
       <c r="C96">
-        <v>103000</v>
+        <v>1238</v>
       </c>
     </row>
     <row r="97" spans="1:3">
@@ -1442,7 +1468,7 @@
         <v>3</v>
       </c>
       <c r="C97">
-        <v>44000</v>
+        <v>998</v>
       </c>
     </row>
     <row r="98" spans="1:3">
@@ -1453,7 +1479,7 @@
         <v>7</v>
       </c>
       <c r="C98">
-        <v>314000</v>
+        <v>1701</v>
       </c>
     </row>
     <row r="99" spans="1:3">
@@ -1464,7 +1490,7 @@
         <v>6</v>
       </c>
       <c r="C99">
-        <v>460000</v>
+        <v>956</v>
       </c>
     </row>
     <row r="100" spans="1:3">
@@ -1475,7 +1501,7 @@
         <v>4</v>
       </c>
       <c r="C100">
-        <v>58000</v>
+        <v>1462</v>
       </c>
     </row>
     <row r="101" spans="1:3">
@@ -1486,7 +1512,7 @@
         <v>8</v>
       </c>
       <c r="C101">
-        <v>50000</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="102" spans="1:3">
@@ -1497,7 +1523,7 @@
         <v>6</v>
       </c>
       <c r="C102">
-        <v>245000</v>
+        <v>662</v>
       </c>
     </row>
     <row r="103" spans="1:3">
@@ -1508,7 +1534,7 @@
         <v>7</v>
       </c>
       <c r="C103">
-        <v>354000</v>
+        <v>953</v>
       </c>
     </row>
     <row r="104" spans="1:3">
@@ -1519,7 +1545,7 @@
         <v>3</v>
       </c>
       <c r="C104">
-        <v>46000</v>
+        <v>1531</v>
       </c>
     </row>
     <row r="105" spans="1:3">
@@ -1530,7 +1556,7 @@
         <v>3</v>
       </c>
       <c r="C105">
-        <v>84000</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="106" spans="1:3">
@@ -1541,7 +1567,7 @@
         <v>8</v>
       </c>
       <c r="C106">
-        <v>50000</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="107" spans="1:3">
@@ -1552,7 +1578,7 @@
         <v>6</v>
       </c>
       <c r="C107">
-        <v>148000</v>
+        <v>831</v>
       </c>
     </row>
     <row r="108" spans="1:3">
@@ -1563,7 +1589,7 @@
         <v>4</v>
       </c>
       <c r="C108">
-        <v>217000</v>
+        <v>235</v>
       </c>
     </row>
     <row r="109" spans="1:3">
@@ -1574,7 +1600,7 @@
         <v>5</v>
       </c>
       <c r="C109">
-        <v>147000</v>
+        <v>804</v>
       </c>
     </row>
     <row r="110" spans="1:3">
@@ -1585,7 +1611,7 @@
         <v>8</v>
       </c>
       <c r="C110">
-        <v>60000</v>
+        <v>217</v>
       </c>
     </row>
     <row r="111" spans="1:3">
@@ -1596,7 +1622,7 @@
         <v>5</v>
       </c>
       <c r="C111">
-        <v>137000</v>
+        <v>90</v>
       </c>
     </row>
     <row r="112" spans="1:3">
@@ -1607,7 +1633,7 @@
         <v>3</v>
       </c>
       <c r="C112">
-        <v>66000</v>
+        <v>173</v>
       </c>
     </row>
     <row r="113" spans="1:3">
@@ -1618,7 +1644,7 @@
         <v>7</v>
       </c>
       <c r="C113">
-        <v>351000</v>
+        <v>1592</v>
       </c>
     </row>
     <row r="114" spans="1:3">
@@ -1629,7 +1655,7 @@
         <v>8</v>
       </c>
       <c r="C114">
-        <v>27000</v>
+        <v>1373</v>
       </c>
     </row>
     <row r="115" spans="1:3">
@@ -1640,7 +1666,7 @@
         <v>9</v>
       </c>
       <c r="C115">
-        <v>1510000</v>
+        <v>229</v>
       </c>
     </row>
     <row r="116" spans="1:3">
@@ -1651,7 +1677,7 @@
         <v>6</v>
       </c>
       <c r="C116">
-        <v>421000</v>
+        <v>1237</v>
       </c>
     </row>
     <row r="117" spans="1:3">
@@ -1662,7 +1688,7 @@
         <v>3</v>
       </c>
       <c r="C117">
-        <v>173000</v>
+        <v>491</v>
       </c>
     </row>
     <row r="118" spans="1:3">
@@ -1673,7 +1699,7 @@
         <v>4</v>
       </c>
       <c r="C118">
-        <v>187000</v>
+        <v>1956</v>
       </c>
     </row>
     <row r="119" spans="1:3">
@@ -1684,7 +1710,7 @@
         <v>5</v>
       </c>
       <c r="C119">
-        <v>87000</v>
+        <v>1778</v>
       </c>
     </row>
     <row r="120" spans="1:3">
@@ -1695,7 +1721,7 @@
         <v>6</v>
       </c>
       <c r="C120">
-        <v>422000</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="121" spans="1:3">
@@ -1706,7 +1732,7 @@
         <v>9</v>
       </c>
       <c r="C121">
-        <v>2894000</v>
+        <v>924</v>
       </c>
     </row>
     <row r="122" spans="1:3">
@@ -1717,7 +1743,7 @@
         <v>8</v>
       </c>
       <c r="C122">
-        <v>64000</v>
+        <v>1810</v>
       </c>
     </row>
     <row r="123" spans="1:3">
@@ -1728,7 +1754,7 @@
         <v>3</v>
       </c>
       <c r="C123">
-        <v>179000</v>
+        <v>532</v>
       </c>
     </row>
     <row r="124" spans="1:3">
@@ -1739,7 +1765,7 @@
         <v>4</v>
       </c>
       <c r="C124">
-        <v>152000</v>
+        <v>614</v>
       </c>
     </row>
     <row r="125" spans="1:3">
@@ -1750,7 +1776,7 @@
         <v>3</v>
       </c>
       <c r="C125">
-        <v>122000</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="126" spans="1:3">
@@ -1761,7 +1787,7 @@
         <v>8</v>
       </c>
       <c r="C126">
-        <v>38000</v>
+        <v>1601</v>
       </c>
     </row>
     <row r="127" spans="1:3">
@@ -1772,7 +1798,7 @@
         <v>9</v>
       </c>
       <c r="C127">
-        <v>1066000</v>
+        <v>1929</v>
       </c>
     </row>
     <row r="128" spans="1:3">
@@ -1783,7 +1809,7 @@
         <v>6</v>
       </c>
       <c r="C128">
-        <v>300000</v>
+        <v>1787</v>
       </c>
     </row>
     <row r="129" spans="1:3">
@@ -1794,7 +1820,7 @@
         <v>9</v>
       </c>
       <c r="C129">
-        <v>2521000</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="130" spans="1:3">
@@ -1805,7 +1831,7 @@
         <v>7</v>
       </c>
       <c r="C130">
-        <v>173000</v>
+        <v>1485</v>
       </c>
     </row>
     <row r="131" spans="1:3">
@@ -1816,7 +1842,7 @@
         <v>5</v>
       </c>
       <c r="C131">
-        <v>32000</v>
+        <v>1570</v>
       </c>
     </row>
     <row r="132" spans="1:3">
@@ -1827,7 +1853,7 @@
         <v>8</v>
       </c>
       <c r="C132">
-        <v>24000</v>
+        <v>1769</v>
       </c>
     </row>
     <row r="133" spans="1:3">
@@ -1838,7 +1864,7 @@
         <v>4</v>
       </c>
       <c r="C133">
-        <v>89000</v>
+        <v>1631</v>
       </c>
     </row>
     <row r="134" spans="1:3">
@@ -1849,7 +1875,7 @@
         <v>3</v>
       </c>
       <c r="C134">
-        <v>190000</v>
+        <v>695</v>
       </c>
     </row>
     <row r="135" spans="1:3">
@@ -1860,7 +1886,7 @@
         <v>5</v>
       </c>
       <c r="C135">
-        <v>60000</v>
+        <v>635</v>
       </c>
     </row>
     <row r="136" spans="1:3">
@@ -1871,7 +1897,7 @@
         <v>4</v>
       </c>
       <c r="C136">
-        <v>252000</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="137" spans="1:3">
@@ -1882,7 +1908,7 @@
         <v>9</v>
       </c>
       <c r="C137">
-        <v>2229000</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="138" spans="1:3">
@@ -1893,7 +1919,7 @@
         <v>9</v>
       </c>
       <c r="C138">
-        <v>2942000</v>
+        <v>1637</v>
       </c>
     </row>
     <row r="139" spans="1:3">
@@ -1904,7 +1930,7 @@
         <v>6</v>
       </c>
       <c r="C139">
-        <v>72000</v>
+        <v>1066</v>
       </c>
     </row>
     <row r="140" spans="1:3">
@@ -1915,7 +1941,7 @@
         <v>5</v>
       </c>
       <c r="C140">
-        <v>118000</v>
+        <v>1516</v>
       </c>
     </row>
     <row r="141" spans="1:3">
@@ -1926,7 +1952,7 @@
         <v>8</v>
       </c>
       <c r="C141">
-        <v>58000</v>
+        <v>44</v>
       </c>
     </row>
     <row r="142" spans="1:3">
@@ -1937,7 +1963,7 @@
         <v>4</v>
       </c>
       <c r="C142">
-        <v>202000</v>
+        <v>1722</v>
       </c>
     </row>
     <row r="143" spans="1:3">
@@ -1948,7 +1974,7 @@
         <v>3</v>
       </c>
       <c r="C143">
-        <v>149000</v>
+        <v>1518</v>
       </c>
     </row>
     <row r="144" spans="1:3">
@@ -1959,7 +1985,7 @@
         <v>3</v>
       </c>
       <c r="C144">
-        <v>165000</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="145" spans="1:3">
@@ -1970,7 +1996,7 @@
         <v>6</v>
       </c>
       <c r="C145">
-        <v>168000</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="146" spans="1:3">
@@ -1981,7 +2007,7 @@
         <v>3</v>
       </c>
       <c r="C146">
-        <v>171000</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="147" spans="1:3">
@@ -1992,7 +2018,7 @@
         <v>8</v>
       </c>
       <c r="C147">
-        <v>11000</v>
+        <v>566</v>
       </c>
     </row>
     <row r="148" spans="1:3">
@@ -2003,7 +2029,7 @@
         <v>5</v>
       </c>
       <c r="C148">
-        <v>49000</v>
+        <v>380</v>
       </c>
     </row>
     <row r="149" spans="1:3">
@@ -2014,7 +2040,7 @@
         <v>5</v>
       </c>
       <c r="C149">
-        <v>88000</v>
+        <v>1506</v>
       </c>
     </row>
     <row r="150" spans="1:3">
@@ -2025,7 +2051,7 @@
         <v>9</v>
       </c>
       <c r="C150">
-        <v>1893000</v>
+        <v>20</v>
       </c>
     </row>
     <row r="151" spans="1:3">
@@ -2036,7 +2062,7 @@
         <v>5</v>
       </c>
       <c r="C151">
-        <v>48000</v>
+        <v>337</v>
       </c>
     </row>
     <row r="152" spans="1:3">
@@ -2047,7 +2073,7 @@
         <v>5</v>
       </c>
       <c r="C152">
-        <v>95000</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="153" spans="1:3">
@@ -2058,7 +2084,7 @@
         <v>9</v>
       </c>
       <c r="C153">
-        <v>2280000</v>
+        <v>673</v>
       </c>
     </row>
     <row r="154" spans="1:3">
@@ -2069,7 +2095,7 @@
         <v>4</v>
       </c>
       <c r="C154">
-        <v>90000</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="155" spans="1:3">
@@ -2080,7 +2106,7 @@
         <v>9</v>
       </c>
       <c r="C155">
-        <v>2358000</v>
+        <v>1195</v>
       </c>
     </row>
     <row r="156" spans="1:3">
@@ -2091,7 +2117,7 @@
         <v>5</v>
       </c>
       <c r="C156">
-        <v>20000</v>
+        <v>178</v>
       </c>
     </row>
     <row r="157" spans="1:3">
@@ -2102,7 +2128,7 @@
         <v>5</v>
       </c>
       <c r="C157">
-        <v>87000</v>
+        <v>1183</v>
       </c>
     </row>
     <row r="158" spans="1:3">
@@ -2113,7 +2139,7 @@
         <v>6</v>
       </c>
       <c r="C158">
-        <v>296000</v>
+        <v>1289</v>
       </c>
     </row>
     <row r="159" spans="1:3">
@@ -2124,7 +2150,7 @@
         <v>5</v>
       </c>
       <c r="C159">
-        <v>65000</v>
+        <v>235</v>
       </c>
     </row>
     <row r="160" spans="1:3">
@@ -2135,7 +2161,7 @@
         <v>7</v>
       </c>
       <c r="C160">
-        <v>599000</v>
+        <v>21</v>
       </c>
     </row>
     <row r="161" spans="1:3">
@@ -2146,7 +2172,7 @@
         <v>7</v>
       </c>
       <c r="C161">
-        <v>188000</v>
+        <v>124</v>
       </c>
     </row>
     <row r="162" spans="1:3">
@@ -2157,7 +2183,7 @@
         <v>9</v>
       </c>
       <c r="C162">
-        <v>1722000</v>
+        <v>1153</v>
       </c>
     </row>
     <row r="163" spans="1:3">
@@ -2168,7 +2194,7 @@
         <v>8</v>
       </c>
       <c r="C163">
-        <v>74000</v>
+        <v>1765</v>
       </c>
     </row>
     <row r="164" spans="1:3">
@@ -2179,7 +2205,7 @@
         <v>6</v>
       </c>
       <c r="C164">
-        <v>351000</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="165" spans="1:3">
@@ -2190,7 +2216,7 @@
         <v>7</v>
       </c>
       <c r="C165">
-        <v>283000</v>
+        <v>1497</v>
       </c>
     </row>
     <row r="166" spans="1:3">
@@ -2201,7 +2227,7 @@
         <v>6</v>
       </c>
       <c r="C166">
-        <v>118000</v>
+        <v>848</v>
       </c>
     </row>
     <row r="167" spans="1:3">
@@ -2212,7 +2238,7 @@
         <v>8</v>
       </c>
       <c r="C167">
-        <v>57000</v>
+        <v>924</v>
       </c>
     </row>
     <row r="168" spans="1:3">
@@ -2223,7 +2249,7 @@
         <v>7</v>
       </c>
       <c r="C168">
-        <v>245000</v>
+        <v>903</v>
       </c>
     </row>
     <row r="169" spans="1:3">
@@ -2234,7 +2260,7 @@
         <v>8</v>
       </c>
       <c r="C169">
-        <v>79000</v>
+        <v>376</v>
       </c>
     </row>
     <row r="170" spans="1:3">
@@ -2245,7 +2271,7 @@
         <v>6</v>
       </c>
       <c r="C170">
-        <v>438000</v>
+        <v>669</v>
       </c>
     </row>
     <row r="171" spans="1:3">
@@ -2256,7 +2282,7 @@
         <v>8</v>
       </c>
       <c r="C171">
-        <v>77000</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="172" spans="1:3">
@@ -2267,7 +2293,7 @@
         <v>5</v>
       </c>
       <c r="C172">
-        <v>20000</v>
+        <v>808</v>
       </c>
     </row>
     <row r="173" spans="1:3">
@@ -2278,7 +2304,7 @@
         <v>3</v>
       </c>
       <c r="C173">
-        <v>183000</v>
+        <v>1289</v>
       </c>
     </row>
     <row r="174" spans="1:3">
@@ -2289,7 +2315,7 @@
         <v>7</v>
       </c>
       <c r="C174">
-        <v>411000</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="175" spans="1:3">
@@ -2300,7 +2326,7 @@
         <v>5</v>
       </c>
       <c r="C175">
-        <v>145000</v>
+        <v>1623</v>
       </c>
     </row>
     <row r="176" spans="1:3">
@@ -2311,7 +2337,7 @@
         <v>6</v>
       </c>
       <c r="C176">
-        <v>49000</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="177" spans="1:3">
@@ -2322,7 +2348,7 @@
         <v>7</v>
       </c>
       <c r="C177">
-        <v>194000</v>
+        <v>1485</v>
       </c>
     </row>
     <row r="178" spans="1:3">
@@ -2333,7 +2359,7 @@
         <v>3</v>
       </c>
       <c r="C178">
-        <v>122000</v>
+        <v>1624</v>
       </c>
     </row>
     <row r="179" spans="1:3">
@@ -2344,7 +2370,7 @@
         <v>7</v>
       </c>
       <c r="C179">
-        <v>394000</v>
+        <v>988</v>
       </c>
     </row>
     <row r="180" spans="1:3">
@@ -2355,7 +2381,7 @@
         <v>4</v>
       </c>
       <c r="C180">
-        <v>111000</v>
+        <v>771</v>
       </c>
     </row>
     <row r="181" spans="1:3">
@@ -2366,7 +2392,7 @@
         <v>3</v>
       </c>
       <c r="C181">
-        <v>44000</v>
+        <v>1492</v>
       </c>
     </row>
     <row r="182" spans="1:3">
@@ -2377,7 +2403,7 @@
         <v>3</v>
       </c>
       <c r="C182">
-        <v>91000</v>
+        <v>913</v>
       </c>
     </row>
     <row r="183" spans="1:3">
@@ -2388,7 +2414,7 @@
         <v>7</v>
       </c>
       <c r="C183">
-        <v>660000</v>
+        <v>386</v>
       </c>
     </row>
     <row r="184" spans="1:3">
@@ -2399,7 +2425,7 @@
         <v>3</v>
       </c>
       <c r="C184">
-        <v>50000</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="185" spans="1:3">
@@ -2410,7 +2436,7 @@
         <v>3</v>
       </c>
       <c r="C185">
-        <v>51000</v>
+        <v>850</v>
       </c>
     </row>
     <row r="186" spans="1:3">
@@ -2421,7 +2447,7 @@
         <v>7</v>
       </c>
       <c r="C186">
-        <v>577000</v>
+        <v>42</v>
       </c>
     </row>
     <row r="187" spans="1:3">
@@ -2432,7 +2458,7 @@
         <v>6</v>
       </c>
       <c r="C187">
-        <v>457000</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="188" spans="1:3">
@@ -2443,7 +2469,7 @@
         <v>6</v>
       </c>
       <c r="C188">
-        <v>75000</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="189" spans="1:3">
@@ -2454,7 +2480,7 @@
         <v>6</v>
       </c>
       <c r="C189">
-        <v>429000</v>
+        <v>44</v>
       </c>
     </row>
     <row r="190" spans="1:3">
@@ -2465,7 +2491,7 @@
         <v>8</v>
       </c>
       <c r="C190">
-        <v>78000</v>
+        <v>1770</v>
       </c>
     </row>
     <row r="191" spans="1:3">
@@ -2476,7 +2502,7 @@
         <v>7</v>
       </c>
       <c r="C191">
-        <v>208000</v>
+        <v>887</v>
       </c>
     </row>
     <row r="192" spans="1:3">
@@ -2487,7 +2513,7 @@
         <v>8</v>
       </c>
       <c r="C192">
-        <v>26000</v>
+        <v>1352</v>
       </c>
     </row>
     <row r="193" spans="1:3">
@@ -2498,7 +2524,7 @@
         <v>9</v>
       </c>
       <c r="C193">
-        <v>2446000</v>
+        <v>1860</v>
       </c>
     </row>
     <row r="194" spans="1:3">
@@ -2509,7 +2535,7 @@
         <v>3</v>
       </c>
       <c r="C194">
-        <v>170000</v>
+        <v>1246</v>
       </c>
     </row>
     <row r="195" spans="1:3">
@@ -2520,7 +2546,7 @@
         <v>6</v>
       </c>
       <c r="C195">
-        <v>124000</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="196" spans="1:3">
@@ -2531,7 +2557,7 @@
         <v>9</v>
       </c>
       <c r="C196">
-        <v>1585000</v>
+        <v>956</v>
       </c>
     </row>
     <row r="197" spans="1:3">
@@ -2542,7 +2568,7 @@
         <v>8</v>
       </c>
       <c r="C197">
-        <v>77000</v>
+        <v>1213</v>
       </c>
     </row>
     <row r="198" spans="1:3">
@@ -2553,7 +2579,7 @@
         <v>7</v>
       </c>
       <c r="C198">
-        <v>701000</v>
+        <v>1953</v>
       </c>
     </row>
     <row r="199" spans="1:3">
@@ -2564,7 +2590,7 @@
         <v>9</v>
       </c>
       <c r="C199">
-        <v>2233000</v>
+        <v>922</v>
       </c>
     </row>
     <row r="200" spans="1:3">
@@ -2575,7 +2601,7 @@
         <v>6</v>
       </c>
       <c r="C200">
-        <v>148000</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="201" spans="1:3">
@@ -2586,7 +2612,7 @@
         <v>8</v>
       </c>
       <c r="C201">
-        <v>79000</v>
+        <v>413</v>
       </c>
     </row>
     <row r="202" spans="1:3">
@@ -2597,7 +2623,7 @@
         <v>4</v>
       </c>
       <c r="C202">
-        <v>243000</v>
+        <v>1441</v>
       </c>
     </row>
     <row r="203" spans="1:3">
@@ -2608,7 +2634,7 @@
         <v>5</v>
       </c>
       <c r="C203">
-        <v>71000</v>
+        <v>1410</v>
       </c>
     </row>
     <row r="204" spans="1:3">
@@ -2619,7 +2645,7 @@
         <v>4</v>
       </c>
       <c r="C204">
-        <v>232000</v>
+        <v>252</v>
       </c>
     </row>
     <row r="205" spans="1:3">
@@ -2630,7 +2656,7 @@
         <v>9</v>
       </c>
       <c r="C205">
-        <v>1776000</v>
+        <v>443</v>
       </c>
     </row>
     <row r="206" spans="1:3">
@@ -2641,7 +2667,7 @@
         <v>8</v>
       </c>
       <c r="C206">
-        <v>61000</v>
+        <v>675</v>
       </c>
     </row>
     <row r="207" spans="1:3">
@@ -2652,7 +2678,7 @@
         <v>9</v>
       </c>
       <c r="C207">
-        <v>2029000</v>
+        <v>631</v>
       </c>
     </row>
     <row r="208" spans="1:3">
@@ -2663,7 +2689,7 @@
         <v>3</v>
       </c>
       <c r="C208">
-        <v>142000</v>
+        <v>279</v>
       </c>
     </row>
     <row r="209" spans="1:3">
@@ -2674,7 +2700,7 @@
         <v>8</v>
       </c>
       <c r="C209">
-        <v>76000</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="210" spans="1:3">
@@ -2685,7 +2711,7 @@
         <v>7</v>
       </c>
       <c r="C210">
-        <v>542000</v>
+        <v>1463</v>
       </c>
     </row>
     <row r="211" spans="1:3">
@@ -2696,7 +2722,7 @@
         <v>9</v>
       </c>
       <c r="C211">
-        <v>995000</v>
+        <v>918</v>
       </c>
     </row>
     <row r="212" spans="1:3">
@@ -2707,7 +2733,7 @@
         <v>7</v>
       </c>
       <c r="C212">
-        <v>333000</v>
+        <v>1622</v>
       </c>
     </row>
     <row r="213" spans="1:3">
@@ -2718,7 +2744,7 @@
         <v>6</v>
       </c>
       <c r="C213">
-        <v>155000</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="214" spans="1:3">
@@ -2729,7 +2755,7 @@
         <v>5</v>
       </c>
       <c r="C214">
-        <v>36000</v>
+        <v>867</v>
       </c>
     </row>
     <row r="215" spans="1:3">
@@ -2740,7 +2766,7 @@
         <v>6</v>
       </c>
       <c r="C215">
-        <v>213000</v>
+        <v>1822</v>
       </c>
     </row>
     <row r="216" spans="1:3">
@@ -2751,7 +2777,7 @@
         <v>9</v>
       </c>
       <c r="C216">
-        <v>586000</v>
+        <v>1805</v>
       </c>
     </row>
     <row r="217" spans="1:3">
@@ -2762,7 +2788,7 @@
         <v>4</v>
       </c>
       <c r="C217">
-        <v>200000</v>
+        <v>257</v>
       </c>
     </row>
     <row r="218" spans="1:3">
@@ -2773,7 +2799,7 @@
         <v>4</v>
       </c>
       <c r="C218">
-        <v>191000</v>
+        <v>1870</v>
       </c>
     </row>
     <row r="219" spans="1:3">
@@ -2784,7 +2810,7 @@
         <v>8</v>
       </c>
       <c r="C219">
-        <v>39000</v>
+        <v>565</v>
       </c>
     </row>
     <row r="220" spans="1:3">
@@ -2795,7 +2821,7 @@
         <v>3</v>
       </c>
       <c r="C220">
-        <v>180000</v>
+        <v>68</v>
       </c>
     </row>
     <row r="221" spans="1:3">
@@ -2806,7 +2832,7 @@
         <v>9</v>
       </c>
       <c r="C221">
-        <v>1402000</v>
+        <v>896</v>
       </c>
     </row>
     <row r="222" spans="1:3">
@@ -2817,7 +2843,7 @@
         <v>5</v>
       </c>
       <c r="C222">
-        <v>21000</v>
+        <v>117</v>
       </c>
     </row>
     <row r="223" spans="1:3">
@@ -2828,7 +2854,7 @@
         <v>5</v>
       </c>
       <c r="C223">
-        <v>38000</v>
+        <v>1193</v>
       </c>
     </row>
     <row r="224" spans="1:3">
@@ -2839,7 +2865,7 @@
         <v>6</v>
       </c>
       <c r="C224">
-        <v>402000</v>
+        <v>1969</v>
       </c>
     </row>
     <row r="225" spans="1:3">
@@ -2850,7 +2876,7 @@
         <v>7</v>
       </c>
       <c r="C225">
-        <v>726000</v>
+        <v>1905</v>
       </c>
     </row>
     <row r="226" spans="1:3">
@@ -2861,7 +2887,7 @@
         <v>4</v>
       </c>
       <c r="C226">
-        <v>65000</v>
+        <v>154</v>
       </c>
     </row>
     <row r="227" spans="1:3">
@@ -2872,7 +2898,7 @@
         <v>7</v>
       </c>
       <c r="C227">
-        <v>314000</v>
+        <v>995</v>
       </c>
     </row>
     <row r="228" spans="1:3">
@@ -2883,7 +2909,7 @@
         <v>8</v>
       </c>
       <c r="C228">
-        <v>18000</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="229" spans="1:3">
@@ -2894,7 +2920,7 @@
         <v>7</v>
       </c>
       <c r="C229">
-        <v>112000</v>
+        <v>1394</v>
       </c>
     </row>
     <row r="230" spans="1:3">
@@ -2905,7 +2931,7 @@
         <v>4</v>
       </c>
       <c r="C230">
-        <v>270000</v>
+        <v>1573</v>
       </c>
     </row>
     <row r="231" spans="1:3">
@@ -2916,7 +2942,7 @@
         <v>3</v>
       </c>
       <c r="C231">
-        <v>114000</v>
+        <v>1936</v>
       </c>
     </row>
     <row r="232" spans="1:3">
@@ -2927,7 +2953,7 @@
         <v>3</v>
       </c>
       <c r="C232">
-        <v>48000</v>
+        <v>475</v>
       </c>
     </row>
     <row r="233" spans="1:3">
@@ -2938,7 +2964,7 @@
         <v>5</v>
       </c>
       <c r="C233">
-        <v>80000</v>
+        <v>243</v>
       </c>
     </row>
     <row r="234" spans="1:3">
@@ -2949,7 +2975,7 @@
         <v>3</v>
       </c>
       <c r="C234">
-        <v>101000</v>
+        <v>1441</v>
       </c>
     </row>
     <row r="235" spans="1:3">
@@ -2960,7 +2986,7 @@
         <v>4</v>
       </c>
       <c r="C235">
-        <v>221000</v>
+        <v>1298</v>
       </c>
     </row>
     <row r="236" spans="1:3">
@@ -2971,7 +2997,7 @@
         <v>5</v>
       </c>
       <c r="C236">
-        <v>144000</v>
+        <v>1749</v>
       </c>
     </row>
     <row r="237" spans="1:3">
@@ -2982,7 +3008,7 @@
         <v>5</v>
       </c>
       <c r="C237">
-        <v>74000</v>
+        <v>537</v>
       </c>
     </row>
     <row r="238" spans="1:3">
@@ -2993,7 +3019,7 @@
         <v>8</v>
       </c>
       <c r="C238">
-        <v>79000</v>
+        <v>1262</v>
       </c>
     </row>
     <row r="239" spans="1:3">
@@ -3004,7 +3030,7 @@
         <v>6</v>
       </c>
       <c r="C239">
-        <v>107000</v>
+        <v>1829</v>
       </c>
     </row>
     <row r="240" spans="1:3">
@@ -3015,7 +3041,7 @@
         <v>8</v>
       </c>
       <c r="C240">
-        <v>70000</v>
+        <v>1458</v>
       </c>
     </row>
     <row r="241" spans="1:3">
@@ -3026,7 +3052,7 @@
         <v>8</v>
       </c>
       <c r="C241">
-        <v>41000</v>
+        <v>311</v>
       </c>
     </row>
     <row r="242" spans="1:3">
@@ -3037,7 +3063,7 @@
         <v>6</v>
       </c>
       <c r="C242">
-        <v>441000</v>
+        <v>1829</v>
       </c>
     </row>
     <row r="243" spans="1:3">
@@ -3048,7 +3074,7 @@
         <v>8</v>
       </c>
       <c r="C243">
-        <v>70000</v>
+        <v>387</v>
       </c>
     </row>
     <row r="244" spans="1:3">
@@ -3059,7 +3085,7 @@
         <v>3</v>
       </c>
       <c r="C244">
-        <v>134000</v>
+        <v>1640</v>
       </c>
     </row>
     <row r="245" spans="1:3">
@@ -3070,7 +3096,7 @@
         <v>6</v>
       </c>
       <c r="C245">
-        <v>137000</v>
+        <v>876</v>
       </c>
     </row>
     <row r="246" spans="1:3">
@@ -3081,7 +3107,7 @@
         <v>4</v>
       </c>
       <c r="C246">
-        <v>74000</v>
+        <v>841</v>
       </c>
     </row>
     <row r="247" spans="1:3">
@@ -3092,7 +3118,7 @@
         <v>5</v>
       </c>
       <c r="C247">
-        <v>44000</v>
+        <v>935</v>
       </c>
     </row>
     <row r="248" spans="1:3">
@@ -3103,7 +3129,7 @@
         <v>5</v>
       </c>
       <c r="C248">
-        <v>130000</v>
+        <v>814</v>
       </c>
     </row>
     <row r="249" spans="1:3">
@@ -3114,7 +3140,7 @@
         <v>9</v>
       </c>
       <c r="C249">
-        <v>1951000</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="250" spans="1:3">
@@ -3125,7 +3151,7 @@
         <v>4</v>
       </c>
       <c r="C250">
-        <v>158000</v>
+        <v>283</v>
       </c>
     </row>
     <row r="251" spans="1:3">
@@ -3136,7 +3162,7 @@
         <v>7</v>
       </c>
       <c r="C251">
-        <v>500000</v>
+        <v>1181</v>
       </c>
     </row>
     <row r="252" spans="1:3">
@@ -3147,7 +3173,7 @@
         <v>4</v>
       </c>
       <c r="C252">
-        <v>169000</v>
+        <v>881</v>
       </c>
     </row>
     <row r="253" spans="1:3">
@@ -3158,7 +3184,7 @@
         <v>6</v>
       </c>
       <c r="C253">
-        <v>482000</v>
+        <v>1946</v>
       </c>
     </row>
     <row r="254" spans="1:3">
@@ -3169,7 +3195,7 @@
         <v>9</v>
       </c>
       <c r="C254">
-        <v>721000</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="255" spans="1:3">
@@ -3180,7 +3206,7 @@
         <v>9</v>
       </c>
       <c r="C255">
-        <v>903000</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="256" spans="1:3">
@@ -3191,7 +3217,7 @@
         <v>4</v>
       </c>
       <c r="C256">
-        <v>65000</v>
+        <v>615</v>
       </c>
     </row>
     <row r="257" spans="1:3">
@@ -3202,7 +3228,7 @@
         <v>7</v>
       </c>
       <c r="C257">
-        <v>492000</v>
+        <v>719</v>
       </c>
     </row>
     <row r="258" spans="1:3">
@@ -3213,7 +3239,7 @@
         <v>7</v>
       </c>
       <c r="C258">
-        <v>427000</v>
+        <v>927</v>
       </c>
     </row>
     <row r="259" spans="1:3">
@@ -3224,7 +3250,7 @@
         <v>8</v>
       </c>
       <c r="C259">
-        <v>23000</v>
+        <v>449</v>
       </c>
     </row>
     <row r="260" spans="1:3">
@@ -3235,7 +3261,7 @@
         <v>5</v>
       </c>
       <c r="C260">
-        <v>83000</v>
+        <v>55</v>
       </c>
     </row>
     <row r="261" spans="1:3">
@@ -3246,7 +3272,7 @@
         <v>4</v>
       </c>
       <c r="C261">
-        <v>99000</v>
+        <v>500</v>
       </c>
     </row>
     <row r="262" spans="1:3">
@@ -3257,7 +3283,7 @@
         <v>7</v>
       </c>
       <c r="C262">
-        <v>274000</v>
+        <v>1402</v>
       </c>
     </row>
     <row r="263" spans="1:3">
@@ -3268,7 +3294,7 @@
         <v>9</v>
       </c>
       <c r="C263">
-        <v>2696000</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="264" spans="1:3">
@@ -3279,7 +3305,7 @@
         <v>5</v>
       </c>
       <c r="C264">
-        <v>134000</v>
+        <v>814</v>
       </c>
     </row>
     <row r="265" spans="1:3">
@@ -3290,7 +3316,7 @@
         <v>5</v>
       </c>
       <c r="C265">
-        <v>55000</v>
+        <v>503</v>
       </c>
     </row>
     <row r="266" spans="1:3">
@@ -3301,7 +3327,7 @@
         <v>6</v>
       </c>
       <c r="C266">
-        <v>256000</v>
+        <v>693</v>
       </c>
     </row>
     <row r="267" spans="1:3">
@@ -3312,7 +3338,7 @@
         <v>7</v>
       </c>
       <c r="C267">
-        <v>267000</v>
+        <v>806</v>
       </c>
     </row>
     <row r="268" spans="1:3">
@@ -3323,7 +3349,7 @@
         <v>4</v>
       </c>
       <c r="C268">
-        <v>121000</v>
+        <v>974</v>
       </c>
     </row>
     <row r="269" spans="1:3">
@@ -3334,7 +3360,7 @@
         <v>7</v>
       </c>
       <c r="C269">
-        <v>553000</v>
+        <v>775</v>
       </c>
     </row>
     <row r="270" spans="1:3">
@@ -3345,7 +3371,7 @@
         <v>5</v>
       </c>
       <c r="C270">
-        <v>83000</v>
+        <v>74</v>
       </c>
     </row>
     <row r="271" spans="1:3">
@@ -3356,7 +3382,7 @@
         <v>9</v>
       </c>
       <c r="C271">
-        <v>808000</v>
+        <v>547</v>
       </c>
     </row>
     <row r="272" spans="1:3">
@@ -3367,7 +3393,7 @@
         <v>8</v>
       </c>
       <c r="C272">
-        <v>66000</v>
+        <v>1026</v>
       </c>
     </row>
     <row r="273" spans="1:3">
@@ -3378,7 +3404,7 @@
         <v>4</v>
       </c>
       <c r="C273">
-        <v>256000</v>
+        <v>1952</v>
       </c>
     </row>
     <row r="274" spans="1:3">
@@ -3389,7 +3415,7 @@
         <v>9</v>
       </c>
       <c r="C274">
-        <v>2754000</v>
+        <v>825</v>
       </c>
     </row>
     <row r="275" spans="1:3">
@@ -3400,7 +3426,7 @@
         <v>8</v>
       </c>
       <c r="C275">
-        <v>22000</v>
+        <v>845</v>
       </c>
     </row>
     <row r="276" spans="1:3">
@@ -3411,7 +3437,7 @@
         <v>4</v>
       </c>
       <c r="C276">
-        <v>62000</v>
+        <v>233</v>
       </c>
     </row>
     <row r="277" spans="1:3">
@@ -3422,7 +3448,7 @@
         <v>6</v>
       </c>
       <c r="C277">
-        <v>373000</v>
+        <v>1044</v>
       </c>
     </row>
     <row r="278" spans="1:3">
@@ -3433,7 +3459,7 @@
         <v>8</v>
       </c>
       <c r="C278">
-        <v>79000</v>
+        <v>1184</v>
       </c>
     </row>
     <row r="279" spans="1:3">
@@ -3444,7 +3470,7 @@
         <v>7</v>
       </c>
       <c r="C279">
-        <v>95000</v>
+        <v>797</v>
       </c>
     </row>
     <row r="280" spans="1:3">
@@ -3455,7 +3481,7 @@
         <v>8</v>
       </c>
       <c r="C280">
-        <v>21000</v>
+        <v>655</v>
       </c>
     </row>
     <row r="281" spans="1:3">
@@ -3466,7 +3492,7 @@
         <v>5</v>
       </c>
       <c r="C281">
-        <v>80000</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="282" spans="1:3">
@@ -3477,7 +3503,7 @@
         <v>5</v>
       </c>
       <c r="C282">
-        <v>62000</v>
+        <v>573</v>
       </c>
     </row>
     <row r="283" spans="1:3">
@@ -3488,7 +3514,7 @@
         <v>7</v>
       </c>
       <c r="C283">
-        <v>496000</v>
+        <v>339</v>
       </c>
     </row>
     <row r="284" spans="1:3">
@@ -3499,7 +3525,7 @@
         <v>8</v>
       </c>
       <c r="C284">
-        <v>72000</v>
+        <v>1506</v>
       </c>
     </row>
     <row r="285" spans="1:3">
@@ -3510,7 +3536,7 @@
         <v>7</v>
       </c>
       <c r="C285">
-        <v>572000</v>
+        <v>1545</v>
       </c>
     </row>
     <row r="286" spans="1:3">
@@ -3521,7 +3547,7 @@
         <v>8</v>
       </c>
       <c r="C286">
-        <v>37000</v>
+        <v>217</v>
       </c>
     </row>
     <row r="287" spans="1:3">
@@ -3532,7 +3558,7 @@
         <v>9</v>
       </c>
       <c r="C287">
-        <v>2142000</v>
+        <v>1548</v>
       </c>
     </row>
     <row r="288" spans="1:3">
@@ -3543,7 +3569,7 @@
         <v>9</v>
       </c>
       <c r="C288">
-        <v>740000</v>
+        <v>1430</v>
       </c>
     </row>
     <row r="289" spans="1:3">
@@ -3554,7 +3580,7 @@
         <v>6</v>
       </c>
       <c r="C289">
-        <v>124000</v>
+        <v>728</v>
       </c>
     </row>
     <row r="290" spans="1:3">
@@ -3565,7 +3591,7 @@
         <v>3</v>
       </c>
       <c r="C290">
-        <v>127000</v>
+        <v>840</v>
       </c>
     </row>
     <row r="291" spans="1:3">
@@ -3576,7 +3602,7 @@
         <v>5</v>
       </c>
       <c r="C291">
-        <v>20000</v>
+        <v>1798</v>
       </c>
     </row>
     <row r="292" spans="1:3">
@@ -3587,7 +3613,7 @@
         <v>7</v>
       </c>
       <c r="C292">
-        <v>479000</v>
+        <v>1414</v>
       </c>
     </row>
     <row r="293" spans="1:3">
@@ -3598,7 +3624,7 @@
         <v>6</v>
       </c>
       <c r="C293">
-        <v>175000</v>
+        <v>228</v>
       </c>
     </row>
     <row r="294" spans="1:3">
@@ -3609,7 +3635,7 @@
         <v>7</v>
       </c>
       <c r="C294">
-        <v>545000</v>
+        <v>196</v>
       </c>
     </row>
     <row r="295" spans="1:3">
@@ -3620,7 +3646,7 @@
         <v>9</v>
       </c>
       <c r="C295">
-        <v>1668000</v>
+        <v>1559</v>
       </c>
     </row>
     <row r="296" spans="1:3">
@@ -3631,7 +3657,7 @@
         <v>6</v>
       </c>
       <c r="C296">
-        <v>256000</v>
+        <v>1563</v>
       </c>
     </row>
     <row r="297" spans="1:3">
@@ -3642,7 +3668,7 @@
         <v>9</v>
       </c>
       <c r="C297">
-        <v>2776000</v>
+        <v>1315</v>
       </c>
     </row>
     <row r="298" spans="1:3">
@@ -3653,7 +3679,7 @@
         <v>7</v>
       </c>
       <c r="C298">
-        <v>757000</v>
+        <v>1741</v>
       </c>
     </row>
     <row r="299" spans="1:3">
@@ -3664,7 +3690,7 @@
         <v>3</v>
       </c>
       <c r="C299">
-        <v>154000</v>
+        <v>356</v>
       </c>
     </row>
     <row r="300" spans="1:3">
@@ -3675,7 +3701,7 @@
         <v>9</v>
       </c>
       <c r="C300">
-        <v>1134000</v>
+        <v>1022</v>
       </c>
     </row>
     <row r="301" spans="1:3">
@@ -3686,7 +3712,7 @@
         <v>3</v>
       </c>
       <c r="C301">
-        <v>78000</v>
+        <v>1168</v>
       </c>
     </row>
     <row r="302" spans="1:3">
@@ -3697,7 +3723,7 @@
         <v>3</v>
       </c>
       <c r="C302">
-        <v>105000</v>
+        <v>1251</v>
       </c>
     </row>
     <row r="303" spans="1:3">
@@ -3708,7 +3734,7 @@
         <v>7</v>
       </c>
       <c r="C303">
-        <v>302000</v>
+        <v>225</v>
       </c>
     </row>
     <row r="304" spans="1:3">
@@ -3719,7 +3745,7 @@
         <v>7</v>
       </c>
       <c r="C304">
-        <v>139000</v>
+        <v>1951</v>
       </c>
     </row>
     <row r="305" spans="1:3">
@@ -3730,7 +3756,7 @@
         <v>8</v>
       </c>
       <c r="C305">
-        <v>79000</v>
+        <v>1941</v>
       </c>
     </row>
     <row r="306" spans="1:3">
@@ -3741,7 +3767,7 @@
         <v>8</v>
       </c>
       <c r="C306">
-        <v>17000</v>
+        <v>1905</v>
       </c>
     </row>
     <row r="307" spans="1:3">
@@ -3752,7 +3778,7 @@
         <v>4</v>
       </c>
       <c r="C307">
-        <v>241000</v>
+        <v>1917</v>
       </c>
     </row>
     <row r="308" spans="1:3">
@@ -3763,7 +3789,7 @@
         <v>8</v>
       </c>
       <c r="C308">
-        <v>50000</v>
+        <v>661</v>
       </c>
     </row>
     <row r="309" spans="1:3">
@@ -3774,7 +3800,7 @@
         <v>7</v>
       </c>
       <c r="C309">
-        <v>138000</v>
+        <v>1994</v>
       </c>
     </row>
     <row r="310" spans="1:3">
@@ -3785,7 +3811,7 @@
         <v>6</v>
       </c>
       <c r="C310">
-        <v>65000</v>
+        <v>1822</v>
       </c>
     </row>
     <row r="311" spans="1:3">
@@ -3796,7 +3822,7 @@
         <v>5</v>
       </c>
       <c r="C311">
-        <v>142000</v>
+        <v>1651</v>
       </c>
     </row>
     <row r="312" spans="1:3">
@@ -3807,7 +3833,7 @@
         <v>9</v>
       </c>
       <c r="C312">
-        <v>2559000</v>
+        <v>827</v>
       </c>
     </row>
     <row r="313" spans="1:3">
@@ -3818,7 +3844,7 @@
         <v>5</v>
       </c>
       <c r="C313">
-        <v>60000</v>
+        <v>951</v>
       </c>
     </row>
     <row r="314" spans="1:3">
@@ -3829,7 +3855,7 @@
         <v>4</v>
       </c>
       <c r="C314">
-        <v>64000</v>
+        <v>745</v>
       </c>
     </row>
     <row r="315" spans="1:3">
@@ -3840,7 +3866,7 @@
         <v>4</v>
       </c>
       <c r="C315">
-        <v>295000</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="316" spans="1:3">
@@ -3851,7 +3877,7 @@
         <v>8</v>
       </c>
       <c r="C316">
-        <v>75000</v>
+        <v>1540</v>
       </c>
     </row>
     <row r="317" spans="1:3">
@@ -3862,7 +3888,7 @@
         <v>4</v>
       </c>
       <c r="C317">
-        <v>70000</v>
+        <v>1194</v>
       </c>
     </row>
     <row r="318" spans="1:3">
@@ -3873,7 +3899,7 @@
         <v>4</v>
       </c>
       <c r="C318">
-        <v>267000</v>
+        <v>1279</v>
       </c>
     </row>
     <row r="319" spans="1:3">
@@ -3884,7 +3910,7 @@
         <v>7</v>
       </c>
       <c r="C319">
-        <v>270000</v>
+        <v>27</v>
       </c>
     </row>
     <row r="320" spans="1:3">
@@ -3895,7 +3921,7 @@
         <v>3</v>
       </c>
       <c r="C320">
-        <v>47000</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="321" spans="1:3">
@@ -3906,7 +3932,7 @@
         <v>7</v>
       </c>
       <c r="C321">
-        <v>689000</v>
+        <v>1879</v>
       </c>
     </row>
     <row r="322" spans="1:3">
@@ -3917,7 +3943,7 @@
         <v>4</v>
       </c>
       <c r="C322">
-        <v>67000</v>
+        <v>117</v>
       </c>
     </row>
     <row r="323" spans="1:3">
@@ -3928,7 +3954,7 @@
         <v>4</v>
       </c>
       <c r="C323">
-        <v>222000</v>
+        <v>296</v>
       </c>
     </row>
     <row r="324" spans="1:3">
@@ -3939,7 +3965,7 @@
         <v>8</v>
       </c>
       <c r="C324">
-        <v>40000</v>
+        <v>564</v>
       </c>
     </row>
     <row r="325" spans="1:3">
@@ -3950,7 +3976,7 @@
         <v>5</v>
       </c>
       <c r="C325">
-        <v>123000</v>
+        <v>649</v>
       </c>
     </row>
     <row r="326" spans="1:3">
@@ -3961,7 +3987,7 @@
         <v>8</v>
       </c>
       <c r="C326">
-        <v>25000</v>
+        <v>903</v>
       </c>
     </row>
     <row r="327" spans="1:3">
@@ -3972,7 +3998,7 @@
         <v>6</v>
       </c>
       <c r="C327">
-        <v>495000</v>
+        <v>221</v>
       </c>
     </row>
     <row r="328" spans="1:3">
@@ -3983,7 +4009,7 @@
         <v>5</v>
       </c>
       <c r="C328">
-        <v>83000</v>
+        <v>1546</v>
       </c>
     </row>
     <row r="329" spans="1:3">
@@ -3994,7 +4020,7 @@
         <v>5</v>
       </c>
       <c r="C329">
-        <v>30000</v>
+        <v>1263</v>
       </c>
     </row>
     <row r="330" spans="1:3">
@@ -4005,7 +4031,7 @@
         <v>4</v>
       </c>
       <c r="C330">
-        <v>208000</v>
+        <v>673</v>
       </c>
     </row>
     <row r="331" spans="1:3">
@@ -4016,7 +4042,7 @@
         <v>7</v>
       </c>
       <c r="C331">
-        <v>163000</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="332" spans="1:3">
@@ -4027,7 +4053,7 @@
         <v>8</v>
       </c>
       <c r="C332">
-        <v>63000</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="333" spans="1:3">
@@ -4038,7 +4064,7 @@
         <v>7</v>
       </c>
       <c r="C333">
-        <v>753000</v>
+        <v>885</v>
       </c>
     </row>
     <row r="334" spans="1:3">
@@ -4049,7 +4075,7 @@
         <v>8</v>
       </c>
       <c r="C334">
-        <v>76000</v>
+        <v>973</v>
       </c>
     </row>
     <row r="335" spans="1:3">
@@ -4060,7 +4086,7 @@
         <v>9</v>
       </c>
       <c r="C335">
-        <v>1795000</v>
+        <v>876</v>
       </c>
     </row>
     <row r="336" spans="1:3">
@@ -4071,7 +4097,7 @@
         <v>5</v>
       </c>
       <c r="C336">
-        <v>86000</v>
+        <v>516</v>
       </c>
     </row>
     <row r="337" spans="1:3">
@@ -4082,7 +4108,7 @@
         <v>7</v>
       </c>
       <c r="C337">
-        <v>289000</v>
+        <v>244</v>
       </c>
     </row>
     <row r="338" spans="1:3">
@@ -4093,7 +4119,7 @@
         <v>4</v>
       </c>
       <c r="C338">
-        <v>221000</v>
+        <v>721</v>
       </c>
     </row>
     <row r="339" spans="1:3">
@@ -4104,7 +4130,7 @@
         <v>5</v>
       </c>
       <c r="C339">
-        <v>100000</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="340" spans="1:3">
@@ -4115,7 +4141,7 @@
         <v>7</v>
       </c>
       <c r="C340">
-        <v>324000</v>
+        <v>254</v>
       </c>
     </row>
     <row r="341" spans="1:3">
@@ -4126,7 +4152,7 @@
         <v>6</v>
       </c>
       <c r="C341">
-        <v>175000</v>
+        <v>1765</v>
       </c>
     </row>
     <row r="342" spans="1:3">
@@ -4137,7 +4163,7 @@
         <v>3</v>
       </c>
       <c r="C342">
-        <v>131000</v>
+        <v>257</v>
       </c>
     </row>
     <row r="343" spans="1:3">
@@ -4148,7 +4174,7 @@
         <v>9</v>
       </c>
       <c r="C343">
-        <v>1036000</v>
+        <v>141</v>
       </c>
     </row>
     <row r="344" spans="1:3">
@@ -4159,7 +4185,7 @@
         <v>9</v>
       </c>
       <c r="C344">
-        <v>1728000</v>
+        <v>1504</v>
       </c>
     </row>
     <row r="345" spans="1:3">
@@ -4170,7 +4196,7 @@
         <v>8</v>
       </c>
       <c r="C345">
-        <v>68000</v>
+        <v>343</v>
       </c>
     </row>
     <row r="346" spans="1:3">
@@ -4181,7 +4207,7 @@
         <v>9</v>
       </c>
       <c r="C346">
-        <v>1795000</v>
+        <v>553</v>
       </c>
     </row>
     <row r="347" spans="1:3">
@@ -4192,7 +4218,7 @@
         <v>6</v>
       </c>
       <c r="C347">
-        <v>424000</v>
+        <v>37</v>
       </c>
     </row>
     <row r="348" spans="1:3">
@@ -4203,7 +4229,7 @@
         <v>3</v>
       </c>
       <c r="C348">
-        <v>48000</v>
+        <v>1816</v>
       </c>
     </row>
     <row r="349" spans="1:3">
@@ -4214,7 +4240,7 @@
         <v>7</v>
       </c>
       <c r="C349">
-        <v>89000</v>
+        <v>442</v>
       </c>
     </row>
     <row r="350" spans="1:3">
@@ -4225,7 +4251,7 @@
         <v>9</v>
       </c>
       <c r="C350">
-        <v>2377000</v>
+        <v>1312</v>
       </c>
     </row>
     <row r="351" spans="1:3">
@@ -4236,7 +4262,7 @@
         <v>6</v>
       </c>
       <c r="C351">
-        <v>358000</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="352" spans="1:3">
@@ -4247,7 +4273,7 @@
         <v>6</v>
       </c>
       <c r="C352">
-        <v>328000</v>
+        <v>976</v>
       </c>
     </row>
     <row r="353" spans="1:3">
@@ -4258,7 +4284,7 @@
         <v>8</v>
       </c>
       <c r="C353">
-        <v>22000</v>
+        <v>187</v>
       </c>
     </row>
     <row r="354" spans="1:3">
@@ -4269,7 +4295,7 @@
         <v>9</v>
       </c>
       <c r="C354">
-        <v>800000</v>
+        <v>1599</v>
       </c>
     </row>
     <row r="355" spans="1:3">
@@ -4280,7 +4306,7 @@
         <v>4</v>
       </c>
       <c r="C355">
-        <v>187000</v>
+        <v>1435</v>
       </c>
     </row>
     <row r="356" spans="1:3">
@@ -4291,7 +4317,7 @@
         <v>7</v>
       </c>
       <c r="C356">
-        <v>298000</v>
+        <v>596</v>
       </c>
     </row>
     <row r="357" spans="1:3">
@@ -4302,7 +4328,7 @@
         <v>6</v>
       </c>
       <c r="C357">
-        <v>299000</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="358" spans="1:3">
@@ -4313,7 +4339,7 @@
         <v>7</v>
       </c>
       <c r="C358">
-        <v>351000</v>
+        <v>801</v>
       </c>
     </row>
     <row r="359" spans="1:3">
@@ -4324,7 +4350,7 @@
         <v>7</v>
       </c>
       <c r="C359">
-        <v>215000</v>
+        <v>383</v>
       </c>
     </row>
     <row r="360" spans="1:3">
@@ -4335,7 +4361,7 @@
         <v>5</v>
       </c>
       <c r="C360">
-        <v>109000</v>
+        <v>313</v>
       </c>
     </row>
     <row r="361" spans="1:3">
@@ -4346,7 +4372,7 @@
         <v>7</v>
       </c>
       <c r="C361">
-        <v>150000</v>
+        <v>688</v>
       </c>
     </row>
     <row r="362" spans="1:3">
@@ -4357,7 +4383,7 @@
         <v>7</v>
       </c>
       <c r="C362">
-        <v>330000</v>
+        <v>624</v>
       </c>
     </row>
     <row r="363" spans="1:3">
@@ -4368,7 +4394,7 @@
         <v>6</v>
       </c>
       <c r="C363">
-        <v>229000</v>
+        <v>420</v>
       </c>
     </row>
     <row r="364" spans="1:3">
@@ -4379,7 +4405,7 @@
         <v>9</v>
       </c>
       <c r="C364">
-        <v>1667000</v>
+        <v>826</v>
       </c>
     </row>
     <row r="365" spans="1:3">
@@ -4390,7 +4416,7 @@
         <v>3</v>
       </c>
       <c r="C365">
-        <v>70000</v>
+        <v>797</v>
       </c>
     </row>
     <row r="366" spans="1:3">
@@ -4401,7 +4427,7 @@
         <v>3</v>
       </c>
       <c r="C366">
-        <v>142000</v>
+        <v>1364</v>
       </c>
     </row>
     <row r="367" spans="1:3">
@@ -4412,7 +4438,7 @@
         <v>6</v>
       </c>
       <c r="C367">
-        <v>466000</v>
+        <v>735</v>
       </c>
     </row>
     <row r="368" spans="1:3">
@@ -4423,7 +4449,7 @@
         <v>6</v>
       </c>
       <c r="C368">
-        <v>318000</v>
+        <v>847</v>
       </c>
     </row>
     <row r="369" spans="1:3">
@@ -4434,7 +4460,7 @@
         <v>3</v>
       </c>
       <c r="C369">
-        <v>107000</v>
+        <v>303</v>
       </c>
     </row>
     <row r="370" spans="1:3">
@@ -4445,7 +4471,7 @@
         <v>7</v>
       </c>
       <c r="C370">
-        <v>706000</v>
+        <v>1585</v>
       </c>
     </row>
     <row r="371" spans="1:3">
@@ -4456,7 +4482,7 @@
         <v>4</v>
       </c>
       <c r="C371">
-        <v>256000</v>
+        <v>580</v>
       </c>
     </row>
     <row r="372" spans="1:3">
@@ -4467,7 +4493,7 @@
         <v>5</v>
       </c>
       <c r="C372">
-        <v>22000</v>
+        <v>359</v>
       </c>
     </row>
     <row r="373" spans="1:3">
@@ -4478,7 +4504,7 @@
         <v>5</v>
       </c>
       <c r="C373">
-        <v>96000</v>
+        <v>437</v>
       </c>
     </row>
     <row r="374" spans="1:3">
@@ -4489,7 +4515,7 @@
         <v>4</v>
       </c>
       <c r="C374">
-        <v>288000</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="375" spans="1:3">
@@ -4500,7 +4526,7 @@
         <v>3</v>
       </c>
       <c r="C375">
-        <v>199000</v>
+        <v>958</v>
       </c>
     </row>
     <row r="376" spans="1:3">
@@ -4511,7 +4537,7 @@
         <v>7</v>
       </c>
       <c r="C376">
-        <v>186000</v>
+        <v>334</v>
       </c>
     </row>
     <row r="377" spans="1:3">
@@ -4522,7 +4548,7 @@
         <v>7</v>
       </c>
       <c r="C377">
-        <v>217000</v>
+        <v>167</v>
       </c>
     </row>
     <row r="378" spans="1:3">
@@ -4533,7 +4559,7 @@
         <v>8</v>
       </c>
       <c r="C378">
-        <v>43000</v>
+        <v>920</v>
       </c>
     </row>
     <row r="379" spans="1:3">
@@ -4544,7 +4570,7 @@
         <v>8</v>
       </c>
       <c r="C379">
-        <v>24000</v>
+        <v>1367</v>
       </c>
     </row>
     <row r="380" spans="1:3">
@@ -4555,7 +4581,7 @@
         <v>3</v>
       </c>
       <c r="C380">
-        <v>57000</v>
+        <v>1984</v>
       </c>
     </row>
     <row r="381" spans="1:3">
@@ -4566,7 +4592,7 @@
         <v>5</v>
       </c>
       <c r="C381">
-        <v>59000</v>
+        <v>500</v>
       </c>
     </row>
     <row r="382" spans="1:3">
@@ -4577,7 +4603,7 @@
         <v>5</v>
       </c>
       <c r="C382">
-        <v>89000</v>
+        <v>175</v>
       </c>
     </row>
     <row r="383" spans="1:3">
@@ -4588,7 +4614,7 @@
         <v>7</v>
       </c>
       <c r="C383">
-        <v>368000</v>
+        <v>1375</v>
       </c>
     </row>
     <row r="384" spans="1:3">
@@ -4599,7 +4625,7 @@
         <v>7</v>
       </c>
       <c r="C384">
-        <v>699000</v>
+        <v>161</v>
       </c>
     </row>
     <row r="385" spans="1:3">
@@ -4610,7 +4636,7 @@
         <v>8</v>
       </c>
       <c r="C385">
-        <v>36000</v>
+        <v>1839</v>
       </c>
     </row>
     <row r="386" spans="1:3">
@@ -4621,7 +4647,7 @@
         <v>6</v>
       </c>
       <c r="C386">
-        <v>407000</v>
+        <v>829</v>
       </c>
     </row>
     <row r="387" spans="1:3">
@@ -4632,7 +4658,7 @@
         <v>4</v>
       </c>
       <c r="C387">
-        <v>137000</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="388" spans="1:3">
@@ -4643,7 +4669,7 @@
         <v>8</v>
       </c>
       <c r="C388">
-        <v>36000</v>
+        <v>828</v>
       </c>
     </row>
     <row r="389" spans="1:3">
@@ -4654,7 +4680,7 @@
         <v>5</v>
       </c>
       <c r="C389">
-        <v>87000</v>
+        <v>901</v>
       </c>
     </row>
     <row r="390" spans="1:3">
@@ -4665,7 +4691,7 @@
         <v>6</v>
       </c>
       <c r="C390">
-        <v>298000</v>
+        <v>46</v>
       </c>
     </row>
     <row r="391" spans="1:3">
@@ -4676,7 +4702,7 @@
         <v>5</v>
       </c>
       <c r="C391">
-        <v>145000</v>
+        <v>208</v>
       </c>
     </row>
     <row r="392" spans="1:3">
@@ -4687,7 +4713,7 @@
         <v>6</v>
       </c>
       <c r="C392">
-        <v>168000</v>
+        <v>95</v>
       </c>
     </row>
     <row r="393" spans="1:3">
@@ -4698,7 +4724,7 @@
         <v>5</v>
       </c>
       <c r="C393">
-        <v>33000</v>
+        <v>1008</v>
       </c>
     </row>
     <row r="394" spans="1:3">
@@ -4709,7 +4735,7 @@
         <v>5</v>
       </c>
       <c r="C394">
-        <v>43000</v>
+        <v>1820</v>
       </c>
     </row>
     <row r="395" spans="1:3">
@@ -4720,7 +4746,7 @@
         <v>9</v>
       </c>
       <c r="C395">
-        <v>2234000</v>
+        <v>462</v>
       </c>
     </row>
     <row r="396" spans="1:3">
@@ -4731,7 +4757,7 @@
         <v>5</v>
       </c>
       <c r="C396">
-        <v>90000</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="397" spans="1:3">
@@ -4742,7 +4768,7 @@
         <v>3</v>
       </c>
       <c r="C397">
-        <v>41000</v>
+        <v>1666</v>
       </c>
     </row>
     <row r="398" spans="1:3">
@@ -4753,7 +4779,7 @@
         <v>4</v>
       </c>
       <c r="C398">
-        <v>50000</v>
+        <v>1666</v>
       </c>
     </row>
     <row r="399" spans="1:3">
@@ -4764,7 +4790,7 @@
         <v>4</v>
       </c>
       <c r="C399">
-        <v>135000</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="400" spans="1:3">
@@ -4775,7 +4801,7 @@
         <v>9</v>
       </c>
       <c r="C400">
-        <v>1035000</v>
+        <v>54</v>
       </c>
     </row>
     <row r="401" spans="1:3">
@@ -4786,7 +4812,7 @@
         <v>3</v>
       </c>
       <c r="C401">
-        <v>193000</v>
+        <v>834</v>
       </c>
     </row>
     <row r="402" spans="1:3">
@@ -4797,7 +4823,7 @@
         <v>3</v>
       </c>
       <c r="C402">
-        <v>97000</v>
+        <v>1728</v>
       </c>
     </row>
     <row r="403" spans="1:3">
@@ -4808,7 +4834,7 @@
         <v>8</v>
       </c>
       <c r="C403">
-        <v>30000</v>
+        <v>187</v>
       </c>
     </row>
     <row r="404" spans="1:3">
@@ -4819,7 +4845,7 @@
         <v>4</v>
       </c>
       <c r="C404">
-        <v>239000</v>
+        <v>1328</v>
       </c>
     </row>
     <row r="405" spans="1:3">
@@ -4830,7 +4856,7 @@
         <v>6</v>
       </c>
       <c r="C405">
-        <v>266000</v>
+        <v>1627</v>
       </c>
     </row>
     <row r="406" spans="1:3">
@@ -4841,7 +4867,7 @@
         <v>5</v>
       </c>
       <c r="C406">
-        <v>129000</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="407" spans="1:3">
@@ -4852,7 +4878,7 @@
         <v>7</v>
       </c>
       <c r="C407">
-        <v>654000</v>
+        <v>170</v>
       </c>
     </row>
     <row r="408" spans="1:3">
@@ -4863,7 +4889,7 @@
         <v>6</v>
       </c>
       <c r="C408">
-        <v>44000</v>
+        <v>1934</v>
       </c>
     </row>
     <row r="409" spans="1:3">
@@ -4874,7 +4900,7 @@
         <v>3</v>
       </c>
       <c r="C409">
-        <v>58000</v>
+        <v>288</v>
       </c>
     </row>
     <row r="410" spans="1:3">
@@ -4885,7 +4911,7 @@
         <v>8</v>
       </c>
       <c r="C410">
-        <v>19000</v>
+        <v>231</v>
       </c>
     </row>
     <row r="411" spans="1:3">
@@ -4896,7 +4922,7 @@
         <v>5</v>
       </c>
       <c r="C411">
-        <v>58000</v>
+        <v>711</v>
       </c>
     </row>
     <row r="412" spans="1:3">
@@ -4907,7 +4933,7 @@
         <v>8</v>
       </c>
       <c r="C412">
-        <v>79000</v>
+        <v>1311</v>
       </c>
     </row>
     <row r="413" spans="1:3">
@@ -4918,7 +4944,7 @@
         <v>7</v>
       </c>
       <c r="C413">
-        <v>116000</v>
+        <v>392</v>
       </c>
     </row>
     <row r="414" spans="1:3">
@@ -4929,7 +4955,7 @@
         <v>8</v>
       </c>
       <c r="C414">
-        <v>57000</v>
+        <v>1879</v>
       </c>
     </row>
     <row r="415" spans="1:3">
@@ -4940,7 +4966,7 @@
         <v>9</v>
       </c>
       <c r="C415">
-        <v>2885000</v>
+        <v>1561</v>
       </c>
     </row>
     <row r="416" spans="1:3">
@@ -4951,7 +4977,7 @@
         <v>6</v>
       </c>
       <c r="C416">
-        <v>322000</v>
+        <v>1550</v>
       </c>
     </row>
     <row r="417" spans="1:3">
@@ -4962,7 +4988,7 @@
         <v>5</v>
       </c>
       <c r="C417">
-        <v>57000</v>
+        <v>1507</v>
       </c>
     </row>
     <row r="418" spans="1:3">
@@ -4973,7 +4999,7 @@
         <v>9</v>
       </c>
       <c r="C418">
-        <v>2260000</v>
+        <v>517</v>
       </c>
     </row>
     <row r="419" spans="1:3">
@@ -4984,7 +5010,7 @@
         <v>5</v>
       </c>
       <c r="C419">
-        <v>52000</v>
+        <v>1307</v>
       </c>
     </row>
     <row r="420" spans="1:3">
@@ -4995,7 +5021,7 @@
         <v>3</v>
       </c>
       <c r="C420">
-        <v>40000</v>
+        <v>392</v>
       </c>
     </row>
     <row r="421" spans="1:3">
@@ -5006,7 +5032,7 @@
         <v>9</v>
       </c>
       <c r="C421">
-        <v>1762000</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="422" spans="1:3">
@@ -5017,7 +5043,7 @@
         <v>4</v>
       </c>
       <c r="C422">
-        <v>143000</v>
+        <v>1825</v>
       </c>
     </row>
     <row r="423" spans="1:3">
@@ -5028,7 +5054,7 @@
         <v>8</v>
       </c>
       <c r="C423">
-        <v>15000</v>
+        <v>1065</v>
       </c>
     </row>
     <row r="424" spans="1:3">
@@ -5039,7 +5065,7 @@
         <v>3</v>
       </c>
       <c r="C424">
-        <v>121000</v>
+        <v>917</v>
       </c>
     </row>
     <row r="425" spans="1:3">
@@ -5050,7 +5076,7 @@
         <v>4</v>
       </c>
       <c r="C425">
-        <v>103000</v>
+        <v>1313</v>
       </c>
     </row>
     <row r="426" spans="1:3">
@@ -5061,7 +5087,7 @@
         <v>8</v>
       </c>
       <c r="C426">
-        <v>41000</v>
+        <v>1926</v>
       </c>
     </row>
     <row r="427" spans="1:3">
@@ -5072,7 +5098,7 @@
         <v>9</v>
       </c>
       <c r="C427">
-        <v>921000</v>
+        <v>271</v>
       </c>
     </row>
     <row r="428" spans="1:3">
@@ -5083,7 +5109,7 @@
         <v>9</v>
       </c>
       <c r="C428">
-        <v>1948000</v>
+        <v>1888</v>
       </c>
     </row>
     <row r="429" spans="1:3">
@@ -5094,7 +5120,7 @@
         <v>7</v>
       </c>
       <c r="C429">
-        <v>653000</v>
+        <v>37</v>
       </c>
     </row>
     <row r="430" spans="1:3">
@@ -5105,7 +5131,7 @@
         <v>8</v>
       </c>
       <c r="C430">
-        <v>62000</v>
+        <v>749</v>
       </c>
     </row>
     <row r="431" spans="1:3">
@@ -5116,7 +5142,7 @@
         <v>7</v>
       </c>
       <c r="C431">
-        <v>715000</v>
+        <v>1367</v>
       </c>
     </row>
     <row r="432" spans="1:3">
@@ -5127,7 +5153,7 @@
         <v>3</v>
       </c>
       <c r="C432">
-        <v>69000</v>
+        <v>102</v>
       </c>
     </row>
     <row r="433" spans="1:3">
@@ -5138,7 +5164,7 @@
         <v>9</v>
       </c>
       <c r="C433">
-        <v>1469000</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="434" spans="1:3">
@@ -5149,7 +5175,7 @@
         <v>7</v>
       </c>
       <c r="C434">
-        <v>246000</v>
+        <v>1524</v>
       </c>
     </row>
     <row r="435" spans="1:3">
@@ -5160,7 +5186,7 @@
         <v>8</v>
       </c>
       <c r="C435">
-        <v>32000</v>
+        <v>1263</v>
       </c>
     </row>
     <row r="436" spans="1:3">
@@ -5171,7 +5197,7 @@
         <v>9</v>
       </c>
       <c r="C436">
-        <v>2188000</v>
+        <v>1195</v>
       </c>
     </row>
     <row r="437" spans="1:3">
@@ -5182,7 +5208,7 @@
         <v>5</v>
       </c>
       <c r="C437">
-        <v>26000</v>
+        <v>1749</v>
       </c>
     </row>
     <row r="438" spans="1:3">
@@ -5193,7 +5219,7 @@
         <v>3</v>
       </c>
       <c r="C438">
-        <v>75000</v>
+        <v>149</v>
       </c>
     </row>
     <row r="439" spans="1:3">
@@ -5204,7 +5230,7 @@
         <v>4</v>
       </c>
       <c r="C439">
-        <v>238000</v>
+        <v>542</v>
       </c>
     </row>
     <row r="440" spans="1:3">
@@ -5215,7 +5241,7 @@
         <v>4</v>
       </c>
       <c r="C440">
-        <v>286000</v>
+        <v>756</v>
       </c>
     </row>
     <row r="441" spans="1:3">
@@ -5226,7 +5252,7 @@
         <v>9</v>
       </c>
       <c r="C441">
-        <v>1860000</v>
+        <v>1906</v>
       </c>
     </row>
     <row r="442" spans="1:3">
@@ -5237,7 +5263,7 @@
         <v>9</v>
       </c>
       <c r="C442">
-        <v>2186000</v>
+        <v>94</v>
       </c>
     </row>
     <row r="443" spans="1:3">
@@ -5248,7 +5274,7 @@
         <v>5</v>
       </c>
       <c r="C443">
-        <v>83000</v>
+        <v>537</v>
       </c>
     </row>
     <row r="444" spans="1:3">
@@ -5259,7 +5285,7 @@
         <v>6</v>
       </c>
       <c r="C444">
-        <v>176000</v>
+        <v>683</v>
       </c>
     </row>
     <row r="445" spans="1:3">
@@ -5270,7 +5296,7 @@
         <v>6</v>
       </c>
       <c r="C445">
-        <v>121000</v>
+        <v>1615</v>
       </c>
     </row>
     <row r="446" spans="1:3">
@@ -5281,7 +5307,7 @@
         <v>5</v>
       </c>
       <c r="C446">
-        <v>47000</v>
+        <v>219</v>
       </c>
     </row>
     <row r="447" spans="1:3">
@@ -5292,7 +5318,7 @@
         <v>4</v>
       </c>
       <c r="C447">
-        <v>147000</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="448" spans="1:3">
@@ -5303,7 +5329,7 @@
         <v>6</v>
       </c>
       <c r="C448">
-        <v>486000</v>
+        <v>1529</v>
       </c>
     </row>
     <row r="449" spans="1:3">
@@ -5314,7 +5340,7 @@
         <v>6</v>
       </c>
       <c r="C449">
-        <v>59000</v>
+        <v>815</v>
       </c>
     </row>
     <row r="450" spans="1:3">
@@ -5325,7 +5351,7 @@
         <v>7</v>
       </c>
       <c r="C450">
-        <v>561000</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="451" spans="1:3">
@@ -5336,7 +5362,7 @@
         <v>9</v>
       </c>
       <c r="C451">
-        <v>1411000</v>
+        <v>1482</v>
       </c>
     </row>
     <row r="452" spans="1:3">
@@ -5347,7 +5373,7 @@
         <v>3</v>
       </c>
       <c r="C452">
-        <v>81000</v>
+        <v>365</v>
       </c>
     </row>
     <row r="453" spans="1:3">
@@ -5358,7 +5384,7 @@
         <v>6</v>
       </c>
       <c r="C453">
-        <v>458000</v>
+        <v>858</v>
       </c>
     </row>
     <row r="454" spans="1:3">
@@ -5369,7 +5395,7 @@
         <v>6</v>
       </c>
       <c r="C454">
-        <v>275000</v>
+        <v>1347</v>
       </c>
     </row>
     <row r="455" spans="1:3">
@@ -5380,7 +5406,7 @@
         <v>6</v>
       </c>
       <c r="C455">
-        <v>219000</v>
+        <v>756</v>
       </c>
     </row>
     <row r="456" spans="1:3">
@@ -5391,7 +5417,7 @@
         <v>6</v>
       </c>
       <c r="C456">
-        <v>196000</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="457" spans="1:3">
@@ -5402,7 +5428,7 @@
         <v>7</v>
       </c>
       <c r="C457">
-        <v>313000</v>
+        <v>552</v>
       </c>
     </row>
     <row r="458" spans="1:3">
@@ -5413,7 +5439,7 @@
         <v>4</v>
       </c>
       <c r="C458">
-        <v>107000</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="459" spans="1:3">
@@ -5424,7 +5450,7 @@
         <v>6</v>
       </c>
       <c r="C459">
-        <v>52000</v>
+        <v>24</v>
       </c>
     </row>
     <row r="460" spans="1:3">
@@ -5435,7 +5461,7 @@
         <v>9</v>
       </c>
       <c r="C460">
-        <v>1291000</v>
+        <v>806</v>
       </c>
     </row>
     <row r="461" spans="1:3">
@@ -5446,7 +5472,7 @@
         <v>5</v>
       </c>
       <c r="C461">
-        <v>122000</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="462" spans="1:3">
@@ -5457,7 +5483,7 @@
         <v>6</v>
       </c>
       <c r="C462">
-        <v>208000</v>
+        <v>1548</v>
       </c>
     </row>
     <row r="463" spans="1:3">
@@ -5468,7 +5494,7 @@
         <v>6</v>
       </c>
       <c r="C463">
-        <v>182000</v>
+        <v>1736</v>
       </c>
     </row>
     <row r="464" spans="1:3">
@@ -5479,7 +5505,7 @@
         <v>4</v>
       </c>
       <c r="C464">
-        <v>271000</v>
+        <v>134</v>
       </c>
     </row>
     <row r="465" spans="1:3">
@@ -5490,7 +5516,7 @@
         <v>3</v>
       </c>
       <c r="C465">
-        <v>47000</v>
+        <v>1926</v>
       </c>
     </row>
     <row r="466" spans="1:3">
@@ -5501,7 +5527,7 @@
         <v>9</v>
       </c>
       <c r="C466">
-        <v>1643000</v>
+        <v>1948</v>
       </c>
     </row>
     <row r="467" spans="1:3">
@@ -5512,7 +5538,7 @@
         <v>7</v>
       </c>
       <c r="C467">
-        <v>439000</v>
+        <v>1543</v>
       </c>
     </row>
     <row r="468" spans="1:3">
@@ -5523,7 +5549,7 @@
         <v>9</v>
       </c>
       <c r="C468">
-        <v>2586000</v>
+        <v>1635</v>
       </c>
     </row>
     <row r="469" spans="1:3">
@@ -5534,7 +5560,7 @@
         <v>4</v>
       </c>
       <c r="C469">
-        <v>152000</v>
+        <v>881</v>
       </c>
     </row>
     <row r="470" spans="1:3">
@@ -5545,7 +5571,7 @@
         <v>5</v>
       </c>
       <c r="C470">
-        <v>104000</v>
+        <v>110</v>
       </c>
     </row>
     <row r="471" spans="1:3">
@@ -5556,7 +5582,7 @@
         <v>9</v>
       </c>
       <c r="C471">
-        <v>613000</v>
+        <v>49</v>
       </c>
     </row>
     <row r="472" spans="1:3">
@@ -5567,7 +5593,7 @@
         <v>6</v>
       </c>
       <c r="C472">
-        <v>99000</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="473" spans="1:3">
@@ -5578,7 +5604,7 @@
         <v>6</v>
       </c>
       <c r="C473">
-        <v>489000</v>
+        <v>768</v>
       </c>
     </row>
     <row r="474" spans="1:3">
@@ -5589,7 +5615,7 @@
         <v>7</v>
       </c>
       <c r="C474">
-        <v>347000</v>
+        <v>1178</v>
       </c>
     </row>
     <row r="475" spans="1:3">
@@ -5600,7 +5626,7 @@
         <v>8</v>
       </c>
       <c r="C475">
-        <v>32000</v>
+        <v>779</v>
       </c>
     </row>
     <row r="476" spans="1:3">
@@ -5611,7 +5637,7 @@
         <v>3</v>
       </c>
       <c r="C476">
-        <v>178000</v>
+        <v>528</v>
       </c>
     </row>
     <row r="477" spans="1:3">
@@ -5622,7 +5648,7 @@
         <v>3</v>
       </c>
       <c r="C477">
-        <v>97000</v>
+        <v>936</v>
       </c>
     </row>
     <row r="478" spans="1:3">
@@ -5633,7 +5659,7 @@
         <v>4</v>
       </c>
       <c r="C478">
-        <v>59000</v>
+        <v>1641</v>
       </c>
     </row>
     <row r="479" spans="1:3">
@@ -5644,7 +5670,7 @@
         <v>3</v>
       </c>
       <c r="C479">
-        <v>57000</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="480" spans="1:3">
@@ -5655,7 +5681,7 @@
         <v>4</v>
       </c>
       <c r="C480">
-        <v>202000</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="481" spans="1:3">
@@ -5666,7 +5692,7 @@
         <v>7</v>
       </c>
       <c r="C481">
-        <v>524000</v>
+        <v>568</v>
       </c>
     </row>
     <row r="482" spans="1:3">
@@ -5677,7 +5703,7 @@
         <v>5</v>
       </c>
       <c r="C482">
-        <v>108000</v>
+        <v>306</v>
       </c>
     </row>
     <row r="483" spans="1:3">
@@ -5688,7 +5714,7 @@
         <v>6</v>
       </c>
       <c r="C483">
-        <v>413000</v>
+        <v>481</v>
       </c>
     </row>
     <row r="484" spans="1:3">
@@ -5699,7 +5725,7 @@
         <v>5</v>
       </c>
       <c r="C484">
-        <v>100000</v>
+        <v>563</v>
       </c>
     </row>
     <row r="485" spans="1:3">
@@ -5710,7 +5736,7 @@
         <v>6</v>
       </c>
       <c r="C485">
-        <v>263000</v>
+        <v>532</v>
       </c>
     </row>
     <row r="486" spans="1:3">
@@ -5721,7 +5747,7 @@
         <v>6</v>
       </c>
       <c r="C486">
-        <v>350000</v>
+        <v>685</v>
       </c>
     </row>
     <row r="487" spans="1:3">
@@ -5732,7 +5758,7 @@
         <v>9</v>
       </c>
       <c r="C487">
-        <v>2594000</v>
+        <v>397</v>
       </c>
     </row>
     <row r="488" spans="1:3">
@@ -5743,7 +5769,7 @@
         <v>7</v>
       </c>
       <c r="C488">
-        <v>198000</v>
+        <v>313</v>
       </c>
     </row>
     <row r="489" spans="1:3">
@@ -5754,7 +5780,7 @@
         <v>9</v>
       </c>
       <c r="C489">
-        <v>2077000</v>
+        <v>560</v>
       </c>
     </row>
     <row r="490" spans="1:3">
@@ -5765,7 +5791,7 @@
         <v>6</v>
       </c>
       <c r="C490">
-        <v>500000</v>
+        <v>818</v>
       </c>
     </row>
     <row r="491" spans="1:3">
@@ -5776,7 +5802,7 @@
         <v>4</v>
       </c>
       <c r="C491">
-        <v>197000</v>
+        <v>879</v>
       </c>
     </row>
     <row r="492" spans="1:3">
@@ -5787,7 +5813,7 @@
         <v>9</v>
       </c>
       <c r="C492">
-        <v>1278000</v>
+        <v>595</v>
       </c>
     </row>
     <row r="493" spans="1:3">
@@ -5798,7 +5824,7 @@
         <v>5</v>
       </c>
       <c r="C493">
-        <v>85000</v>
+        <v>1919</v>
       </c>
     </row>
     <row r="494" spans="1:3">
@@ -5809,7 +5835,7 @@
         <v>5</v>
       </c>
       <c r="C494">
-        <v>31000</v>
+        <v>300</v>
       </c>
     </row>
     <row r="495" spans="1:3">
@@ -5820,7 +5846,7 @@
         <v>8</v>
       </c>
       <c r="C495">
-        <v>65000</v>
+        <v>693</v>
       </c>
     </row>
     <row r="496" spans="1:3">
@@ -5831,7 +5857,7 @@
         <v>8</v>
       </c>
       <c r="C496">
-        <v>10000</v>
+        <v>1111</v>
       </c>
     </row>
     <row r="497" spans="1:3">
@@ -5842,7 +5868,7 @@
         <v>9</v>
       </c>
       <c r="C497">
-        <v>2629000</v>
+        <v>674</v>
       </c>
     </row>
     <row r="498" spans="1:3">
@@ -5853,7 +5879,7 @@
         <v>8</v>
       </c>
       <c r="C498">
-        <v>78000</v>
+        <v>1944</v>
       </c>
     </row>
     <row r="499" spans="1:3">
@@ -5864,7 +5890,7 @@
         <v>7</v>
       </c>
       <c r="C499">
-        <v>783000</v>
+        <v>783</v>
       </c>
     </row>
     <row r="500" spans="1:3">
@@ -5875,7 +5901,7 @@
         <v>5</v>
       </c>
       <c r="C500">
-        <v>70000</v>
+        <v>1704</v>
       </c>
     </row>
     <row r="501" spans="1:3">
@@ -5886,7 +5912,7 @@
         <v>9</v>
       </c>
       <c r="C501">
-        <v>1991000</v>
+        <v>1351</v>
       </c>
     </row>
   </sheetData>

</xml_diff>